<commit_message>
Update researcher role in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -6888,17 +6888,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>researcher</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>An occupational role that is a researcher but unclear what discipline.</t>
+          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>occupational role of source</t>
+          <t>occupational role</t>
         </is>
       </c>
       <c r="E108" s="2" t="n"/>
@@ -7089,7 +7089,7 @@
       <c r="N111" s="2" t="n"/>
       <c r="O111" s="2" t="n"/>
       <c r="P111" s="2" t="n"/>
-      <c r="Q111" s="2" t="inlineStr"/>
+      <c r="Q111" s="2" t="n"/>
       <c r="R111" s="2" t="n"/>
       <c r="S111" s="2" t="n"/>
       <c r="T111" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update researcher in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -6888,7 +6888,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>researcher role</t>
+          <t>researcher</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -6898,7 +6898,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>occupational role</t>
+          <t>occupational role of source</t>
         </is>
       </c>
       <c r="E108" s="2" t="n"/>

</xml_diff>

<commit_message>
Update Label of trainee role in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -535,27 +535,27 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>To be reviewed by</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer query</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Definition_ID</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Curator</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>To be reviewed by</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_ID</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Reviewer query</t>
         </is>
       </c>
     </row>
@@ -601,12 +601,12 @@
         </is>
       </c>
       <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="n"/>
       <c r="Z2" s="2" t="n"/>
@@ -657,12 +657,12 @@
         </is>
       </c>
       <c r="U3" s="2" t="n"/>
-      <c r="V3" s="2" t="n"/>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n"/>
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="n"/>
       <c r="Z3" s="2" t="n"/>
@@ -709,12 +709,12 @@
         </is>
       </c>
       <c r="U4" s="2" t="n"/>
-      <c r="V4" s="2" t="n"/>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="n"/>
       <c r="X4" s="2" t="n"/>
       <c r="Y4" s="2" t="n"/>
       <c r="Z4" s="2" t="n"/>
@@ -769,12 +769,12 @@
         </is>
       </c>
       <c r="U5" s="2" t="n"/>
-      <c r="V5" s="2" t="n"/>
-      <c r="W5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="n"/>
       <c r="X5" s="2" t="n"/>
       <c r="Y5" s="2" t="inlineStr">
         <is>
@@ -833,12 +833,12 @@
         </is>
       </c>
       <c r="U6" s="2" t="n"/>
-      <c r="V6" s="2" t="n"/>
-      <c r="W6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="n"/>
       <c r="X6" s="2" t="n"/>
       <c r="Y6" s="2" t="n"/>
       <c r="Z6" s="2" t="n"/>
@@ -893,12 +893,12 @@
         </is>
       </c>
       <c r="U7" s="2" t="n"/>
-      <c r="V7" s="2" t="n"/>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n"/>
       <c r="X7" s="2" t="n"/>
       <c r="Y7" s="2" t="inlineStr">
         <is>
@@ -957,12 +957,12 @@
         </is>
       </c>
       <c r="U8" s="2" t="n"/>
-      <c r="V8" s="2" t="n"/>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="n"/>
       <c r="X8" s="2" t="n"/>
       <c r="Y8" s="2" t="inlineStr">
         <is>
@@ -1021,12 +1021,12 @@
         </is>
       </c>
       <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="n"/>
-      <c r="W9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="n"/>
       <c r="X9" s="2" t="n"/>
       <c r="Y9" s="2" t="inlineStr">
         <is>
@@ -1081,12 +1081,12 @@
         </is>
       </c>
       <c r="U10" s="2" t="n"/>
-      <c r="V10" s="2" t="n"/>
-      <c r="W10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="n"/>
       <c r="X10" s="2" t="n"/>
       <c r="Y10" s="2" t="inlineStr">
         <is>
@@ -1145,12 +1145,12 @@
         </is>
       </c>
       <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="n"/>
-      <c r="W11" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="n"/>
       <c r="X11" s="2" t="n"/>
       <c r="Y11" s="2" t="inlineStr">
         <is>
@@ -1209,12 +1209,12 @@
         </is>
       </c>
       <c r="U12" s="2" t="n"/>
-      <c r="V12" s="2" t="n"/>
-      <c r="W12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="n"/>
       <c r="X12" s="2" t="n"/>
       <c r="Y12" s="2" t="inlineStr">
         <is>
@@ -1273,12 +1273,12 @@
         </is>
       </c>
       <c r="U13" s="2" t="n"/>
-      <c r="V13" s="2" t="n"/>
-      <c r="W13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="n"/>
       <c r="X13" s="2" t="n"/>
       <c r="Y13" s="2" t="inlineStr">
         <is>
@@ -1331,17 +1331,17 @@
       <c r="U14" s="2" t="n"/>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="W14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="n"/>
       <c r="X14" s="2" t="n"/>
       <c r="Y14" s="2" t="n"/>
-      <c r="Z14" s="2" t="n"/>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1393,12 +1393,12 @@
         </is>
       </c>
       <c r="U15" s="2" t="n"/>
-      <c r="V15" s="2" t="n"/>
-      <c r="W15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="n"/>
       <c r="X15" s="2" t="n"/>
       <c r="Y15" s="2" t="inlineStr">
         <is>
@@ -1453,12 +1453,12 @@
         </is>
       </c>
       <c r="U16" s="2" t="n"/>
-      <c r="V16" s="2" t="n"/>
-      <c r="W16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="n"/>
       <c r="X16" s="2" t="n"/>
       <c r="Y16" s="2" t="n"/>
       <c r="Z16" s="2" t="n"/>
@@ -1513,12 +1513,12 @@
         </is>
       </c>
       <c r="U17" s="2" t="n"/>
-      <c r="V17" s="2" t="n"/>
-      <c r="W17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="n"/>
       <c r="X17" s="2" t="n"/>
       <c r="Y17" s="2" t="inlineStr">
         <is>
@@ -1573,12 +1573,12 @@
         </is>
       </c>
       <c r="U18" s="2" t="n"/>
-      <c r="V18" s="2" t="n"/>
-      <c r="W18" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="n"/>
       <c r="X18" s="2" t="n"/>
       <c r="Y18" s="2" t="n"/>
       <c r="Z18" s="2" t="n"/>
@@ -1633,12 +1633,12 @@
         </is>
       </c>
       <c r="U19" s="2" t="n"/>
-      <c r="V19" s="2" t="n"/>
-      <c r="W19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="n"/>
       <c r="X19" s="2" t="n"/>
       <c r="Y19" s="2" t="inlineStr">
         <is>
@@ -1689,12 +1689,12 @@
         </is>
       </c>
       <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="n"/>
-      <c r="W20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="n"/>
       <c r="X20" s="2" t="n"/>
       <c r="Y20" s="2" t="n"/>
       <c r="Z20" s="2" t="n"/>
@@ -1749,12 +1749,12 @@
         </is>
       </c>
       <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="n"/>
-      <c r="W21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="n"/>
       <c r="X21" s="2" t="n"/>
       <c r="Y21" s="2" t="inlineStr">
         <is>
@@ -1813,12 +1813,12 @@
         </is>
       </c>
       <c r="U22" s="2" t="n"/>
-      <c r="V22" s="2" t="n"/>
-      <c r="W22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="n"/>
       <c r="X22" s="2" t="n"/>
       <c r="Y22" s="2" t="inlineStr">
         <is>
@@ -1877,12 +1877,12 @@
         </is>
       </c>
       <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
-      <c r="W23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="n"/>
       <c r="X23" s="2" t="n"/>
       <c r="Y23" s="2" t="inlineStr">
         <is>
@@ -1941,12 +1941,12 @@
         </is>
       </c>
       <c r="U24" s="2" t="n"/>
-      <c r="V24" s="2" t="n"/>
-      <c r="W24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="n"/>
       <c r="X24" s="2" t="n"/>
       <c r="Y24" s="2" t="inlineStr">
         <is>
@@ -2005,12 +2005,12 @@
         </is>
       </c>
       <c r="U25" s="2" t="n"/>
-      <c r="V25" s="2" t="n"/>
-      <c r="W25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="n"/>
       <c r="X25" s="2" t="n"/>
       <c r="Y25" s="2" t="inlineStr">
         <is>
@@ -2069,12 +2069,12 @@
         </is>
       </c>
       <c r="U26" s="2" t="n"/>
-      <c r="V26" s="2" t="n"/>
-      <c r="W26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="n"/>
       <c r="X26" s="2" t="n"/>
       <c r="Y26" s="2" t="inlineStr">
         <is>
@@ -2131,17 +2131,17 @@
       <c r="U27" s="2" t="n"/>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="n"/>
       <c r="X27" s="2" t="n"/>
       <c r="Y27" s="2" t="n"/>
-      <c r="Z27" s="2" t="n"/>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2193,12 +2193,12 @@
         </is>
       </c>
       <c r="U28" s="2" t="n"/>
-      <c r="V28" s="2" t="n"/>
-      <c r="W28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="n"/>
       <c r="X28" s="2" t="n"/>
       <c r="Y28" s="2" t="n"/>
       <c r="Z28" s="2" t="n"/>
@@ -2249,12 +2249,12 @@
         </is>
       </c>
       <c r="U29" s="2" t="n"/>
-      <c r="V29" s="2" t="n"/>
-      <c r="W29" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="n"/>
       <c r="X29" s="2" t="n"/>
       <c r="Y29" s="2" t="n"/>
       <c r="Z29" s="2" t="n"/>
@@ -2309,12 +2309,12 @@
         </is>
       </c>
       <c r="U30" s="2" t="n"/>
-      <c r="V30" s="2" t="n"/>
-      <c r="W30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="n"/>
       <c r="X30" s="2" t="n"/>
       <c r="Y30" s="2" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
         </is>
       </c>
       <c r="U31" s="2" t="n"/>
-      <c r="V31" s="2" t="n"/>
-      <c r="W31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="n"/>
       <c r="X31" s="2" t="n"/>
       <c r="Y31" s="2" t="inlineStr">
         <is>
@@ -2429,12 +2429,12 @@
         </is>
       </c>
       <c r="U32" s="2" t="n"/>
-      <c r="V32" s="2" t="n"/>
-      <c r="W32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="n"/>
       <c r="X32" s="2" t="n"/>
       <c r="Y32" s="2" t="n"/>
       <c r="Z32" s="2" t="n"/>
@@ -2481,12 +2481,12 @@
         </is>
       </c>
       <c r="U33" s="2" t="n"/>
-      <c r="V33" s="2" t="n"/>
-      <c r="W33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="2" t="n"/>
       <c r="Z33" s="2" t="n"/>
@@ -2541,12 +2541,12 @@
         </is>
       </c>
       <c r="U34" s="2" t="n"/>
-      <c r="V34" s="2" t="n"/>
-      <c r="W34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="n"/>
       <c r="X34" s="2" t="n"/>
       <c r="Y34" s="2" t="inlineStr">
         <is>
@@ -2607,12 +2607,12 @@
         </is>
       </c>
       <c r="U35" s="2" t="n"/>
-      <c r="V35" s="2" t="n"/>
-      <c r="W35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="n"/>
       <c r="X35" s="2" t="n"/>
       <c r="Y35" s="2" t="inlineStr">
         <is>
@@ -2667,12 +2667,12 @@
         </is>
       </c>
       <c r="U36" s="2" t="n"/>
-      <c r="V36" s="2" t="n"/>
-      <c r="W36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="n"/>
       <c r="X36" s="2" t="n"/>
       <c r="Y36" s="2" t="n"/>
       <c r="Z36" s="2" t="n"/>
@@ -2727,12 +2727,12 @@
         </is>
       </c>
       <c r="U37" s="2" t="n"/>
-      <c r="V37" s="2" t="n"/>
-      <c r="W37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="n"/>
       <c r="X37" s="2" t="n"/>
       <c r="Y37" s="2" t="n"/>
       <c r="Z37" s="2" t="n"/>
@@ -2783,12 +2783,12 @@
         </is>
       </c>
       <c r="U38" s="2" t="n"/>
-      <c r="V38" s="2" t="n"/>
-      <c r="W38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="n"/>
       <c r="X38" s="2" t="n"/>
       <c r="Y38" s="2" t="n"/>
       <c r="Z38" s="2" t="n"/>
@@ -2837,17 +2837,17 @@
       <c r="U39" s="2" t="n"/>
       <c r="V39" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W39" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="n"/>
       <c r="X39" s="2" t="n"/>
       <c r="Y39" s="2" t="n"/>
-      <c r="Z39" s="2" t="n"/>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2897,17 +2897,17 @@
       <c r="U40" s="2" t="n"/>
       <c r="V40" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W40" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W40" s="2" t="n"/>
       <c r="X40" s="2" t="n"/>
       <c r="Y40" s="2" t="n"/>
-      <c r="Z40" s="2" t="n"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2959,12 +2959,12 @@
         </is>
       </c>
       <c r="U41" s="2" t="n"/>
-      <c r="V41" s="2" t="n"/>
-      <c r="W41" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V41" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W41" s="2" t="n"/>
       <c r="X41" s="2" t="n"/>
       <c r="Y41" s="2" t="inlineStr">
         <is>
@@ -3015,12 +3015,12 @@
         </is>
       </c>
       <c r="U42" s="2" t="n"/>
-      <c r="V42" s="2" t="n"/>
-      <c r="W42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="n"/>
       <c r="X42" s="2" t="n"/>
       <c r="Y42" s="2" t="n"/>
       <c r="Z42" s="2" t="n"/>
@@ -3069,17 +3069,17 @@
       <c r="U43" s="2" t="n"/>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W43" s="2" t="n"/>
       <c r="X43" s="2" t="n"/>
       <c r="Y43" s="2" t="n"/>
-      <c r="Z43" s="2" t="n"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3127,12 +3127,12 @@
         </is>
       </c>
       <c r="U44" s="2" t="n"/>
-      <c r="V44" s="2" t="n"/>
-      <c r="W44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V44" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W44" s="2" t="n"/>
       <c r="X44" s="2" t="n"/>
       <c r="Y44" s="2" t="n"/>
       <c r="Z44" s="2" t="n"/>
@@ -3187,12 +3187,12 @@
         </is>
       </c>
       <c r="U45" s="2" t="n"/>
-      <c r="V45" s="2" t="n"/>
-      <c r="W45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W45" s="2" t="n"/>
       <c r="X45" s="2" t="n"/>
       <c r="Y45" s="2" t="inlineStr">
         <is>
@@ -3247,12 +3247,12 @@
         </is>
       </c>
       <c r="U46" s="2" t="n"/>
-      <c r="V46" s="2" t="n"/>
-      <c r="W46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V46" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W46" s="2" t="n"/>
       <c r="X46" s="2" t="n"/>
       <c r="Y46" s="2" t="n"/>
       <c r="Z46" s="2" t="n"/>
@@ -3307,12 +3307,12 @@
         </is>
       </c>
       <c r="U47" s="2" t="n"/>
-      <c r="V47" s="2" t="n"/>
-      <c r="W47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W47" s="2" t="n"/>
       <c r="X47" s="2" t="n"/>
       <c r="Y47" s="2" t="inlineStr">
         <is>
@@ -3371,12 +3371,12 @@
         </is>
       </c>
       <c r="U48" s="2" t="n"/>
-      <c r="V48" s="2" t="n"/>
-      <c r="W48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W48" s="2" t="n"/>
       <c r="X48" s="2" t="n"/>
       <c r="Y48" s="2" t="inlineStr">
         <is>
@@ -3435,12 +3435,12 @@
         </is>
       </c>
       <c r="U49" s="2" t="n"/>
-      <c r="V49" s="2" t="n"/>
-      <c r="W49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="n"/>
       <c r="X49" s="2" t="n"/>
       <c r="Y49" s="2" t="inlineStr">
         <is>
@@ -3495,12 +3495,12 @@
         </is>
       </c>
       <c r="U50" s="2" t="n"/>
-      <c r="V50" s="2" t="n"/>
-      <c r="W50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="n"/>
       <c r="X50" s="2" t="n"/>
       <c r="Y50" s="2" t="n"/>
       <c r="Z50" s="2" t="n"/>
@@ -3551,12 +3551,12 @@
         </is>
       </c>
       <c r="U51" s="2" t="n"/>
-      <c r="V51" s="2" t="n"/>
-      <c r="W51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="n"/>
       <c r="X51" s="2" t="n"/>
       <c r="Y51" s="2" t="n"/>
       <c r="Z51" s="2" t="n"/>
@@ -3611,12 +3611,12 @@
         </is>
       </c>
       <c r="U52" s="2" t="n"/>
-      <c r="V52" s="2" t="n"/>
-      <c r="W52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="n"/>
       <c r="X52" s="2" t="n"/>
       <c r="Y52" s="2" t="inlineStr">
         <is>
@@ -3667,12 +3667,12 @@
         </is>
       </c>
       <c r="U53" s="2" t="n"/>
-      <c r="V53" s="2" t="n"/>
-      <c r="W53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V53" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W53" s="2" t="n"/>
       <c r="X53" s="2" t="n"/>
       <c r="Y53" s="2" t="n"/>
       <c r="Z53" s="2" t="n"/>
@@ -3727,12 +3727,12 @@
         </is>
       </c>
       <c r="U54" s="2" t="n"/>
-      <c r="V54" s="2" t="n"/>
-      <c r="W54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="n"/>
       <c r="X54" s="2" t="n"/>
       <c r="Y54" s="2" t="inlineStr">
         <is>
@@ -3787,12 +3787,12 @@
         </is>
       </c>
       <c r="U55" s="2" t="n"/>
-      <c r="V55" s="2" t="n"/>
-      <c r="W55" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W55" s="2" t="n"/>
       <c r="X55" s="2" t="n"/>
       <c r="Y55" s="2" t="n"/>
       <c r="Z55" s="2" t="n"/>
@@ -3843,12 +3843,12 @@
         </is>
       </c>
       <c r="U56" s="2" t="n"/>
-      <c r="V56" s="2" t="n"/>
-      <c r="W56" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="n"/>
       <c r="X56" s="2" t="n"/>
       <c r="Y56" s="2" t="n"/>
       <c r="Z56" s="2" t="n"/>
@@ -3903,12 +3903,12 @@
         </is>
       </c>
       <c r="U57" s="2" t="n"/>
-      <c r="V57" s="2" t="n"/>
-      <c r="W57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="n"/>
       <c r="X57" s="2" t="n"/>
       <c r="Y57" s="2" t="inlineStr">
         <is>
@@ -3967,12 +3967,12 @@
         </is>
       </c>
       <c r="U58" s="2" t="n"/>
-      <c r="V58" s="2" t="n"/>
-      <c r="W58" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="n"/>
       <c r="X58" s="2" t="n"/>
       <c r="Y58" s="2" t="inlineStr">
         <is>
@@ -4027,12 +4027,12 @@
         </is>
       </c>
       <c r="U59" s="2" t="n"/>
-      <c r="V59" s="2" t="n"/>
-      <c r="W59" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="n"/>
       <c r="X59" s="2" t="n"/>
       <c r="Y59" s="2" t="inlineStr">
         <is>
@@ -4091,12 +4091,12 @@
         </is>
       </c>
       <c r="U60" s="2" t="n"/>
-      <c r="V60" s="2" t="n"/>
-      <c r="W60" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V60" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W60" s="2" t="n"/>
       <c r="X60" s="2" t="n"/>
       <c r="Y60" s="2" t="inlineStr">
         <is>
@@ -4151,12 +4151,12 @@
         </is>
       </c>
       <c r="U61" s="2" t="n"/>
-      <c r="V61" s="2" t="n"/>
-      <c r="W61" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W61" s="2" t="n"/>
       <c r="X61" s="2" t="n"/>
       <c r="Y61" s="2" t="n"/>
       <c r="Z61" s="2" t="n"/>
@@ -4209,17 +4209,17 @@
       <c r="U62" s="2" t="n"/>
       <c r="V62" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W62" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="n"/>
       <c r="X62" s="2" t="n"/>
       <c r="Y62" s="2" t="n"/>
-      <c r="Z62" s="2" t="n"/>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4271,12 +4271,12 @@
         </is>
       </c>
       <c r="U63" s="2" t="n"/>
-      <c r="V63" s="2" t="n"/>
-      <c r="W63" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V63" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W63" s="2" t="n"/>
       <c r="X63" s="2" t="n"/>
       <c r="Y63" s="2" t="inlineStr">
         <is>
@@ -4331,12 +4331,12 @@
         </is>
       </c>
       <c r="U64" s="2" t="n"/>
-      <c r="V64" s="2" t="n"/>
-      <c r="W64" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V64" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W64" s="2" t="n"/>
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="2" t="n"/>
       <c r="Z64" s="2" t="n"/>
@@ -4391,12 +4391,12 @@
         </is>
       </c>
       <c r="U65" s="2" t="n"/>
-      <c r="V65" s="2" t="n"/>
-      <c r="W65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V65" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="n"/>
       <c r="X65" s="2" t="n"/>
       <c r="Y65" s="2" t="inlineStr">
         <is>
@@ -4455,12 +4455,12 @@
         </is>
       </c>
       <c r="U66" s="2" t="n"/>
-      <c r="V66" s="2" t="n"/>
-      <c r="W66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V66" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W66" s="2" t="n"/>
       <c r="X66" s="2" t="n"/>
       <c r="Y66" s="2" t="inlineStr">
         <is>
@@ -4519,12 +4519,12 @@
         </is>
       </c>
       <c r="U67" s="2" t="n"/>
-      <c r="V67" s="2" t="n"/>
-      <c r="W67" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W67" s="2" t="n"/>
       <c r="X67" s="2" t="n"/>
       <c r="Y67" s="2" t="inlineStr">
         <is>
@@ -4583,12 +4583,12 @@
         </is>
       </c>
       <c r="U68" s="2" t="n"/>
-      <c r="V68" s="2" t="n"/>
-      <c r="W68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V68" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W68" s="2" t="n"/>
       <c r="X68" s="2" t="n"/>
       <c r="Y68" s="2" t="inlineStr">
         <is>
@@ -4647,12 +4647,12 @@
         </is>
       </c>
       <c r="U69" s="2" t="n"/>
-      <c r="V69" s="2" t="n"/>
-      <c r="W69" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W69" s="2" t="n"/>
       <c r="X69" s="2" t="n"/>
       <c r="Y69" s="2" t="inlineStr">
         <is>
@@ -4707,12 +4707,12 @@
         </is>
       </c>
       <c r="U70" s="2" t="n"/>
-      <c r="V70" s="2" t="n"/>
-      <c r="W70" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V70" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W70" s="2" t="n"/>
       <c r="X70" s="2" t="n"/>
       <c r="Y70" s="2" t="n"/>
       <c r="Z70" s="2" t="n"/>
@@ -4767,12 +4767,12 @@
         </is>
       </c>
       <c r="U71" s="2" t="n"/>
-      <c r="V71" s="2" t="n"/>
-      <c r="W71" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W71" s="2" t="n"/>
       <c r="X71" s="2" t="n"/>
       <c r="Y71" s="2" t="inlineStr">
         <is>
@@ -4827,12 +4827,12 @@
         </is>
       </c>
       <c r="U72" s="2" t="n"/>
-      <c r="V72" s="2" t="n"/>
-      <c r="W72" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V72" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W72" s="2" t="n"/>
       <c r="X72" s="2" t="n"/>
       <c r="Y72" s="2" t="n"/>
       <c r="Z72" s="2" t="n"/>
@@ -4883,12 +4883,12 @@
         </is>
       </c>
       <c r="U73" s="2" t="n"/>
-      <c r="V73" s="2" t="n"/>
-      <c r="W73" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V73" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W73" s="2" t="n"/>
       <c r="X73" s="2" t="n"/>
       <c r="Y73" s="2" t="n"/>
       <c r="Z73" s="2" t="n"/>
@@ -4943,12 +4943,12 @@
         </is>
       </c>
       <c r="U74" s="2" t="n"/>
-      <c r="V74" s="2" t="n"/>
-      <c r="W74" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V74" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W74" s="2" t="n"/>
       <c r="X74" s="2" t="n"/>
       <c r="Y74" s="2" t="inlineStr">
         <is>
@@ -5003,12 +5003,12 @@
         </is>
       </c>
       <c r="U75" s="2" t="n"/>
-      <c r="V75" s="2" t="n"/>
-      <c r="W75" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V75" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W75" s="2" t="n"/>
       <c r="X75" s="2" t="n"/>
       <c r="Y75" s="2" t="inlineStr">
         <is>
@@ -5067,12 +5067,12 @@
         </is>
       </c>
       <c r="U76" s="2" t="n"/>
-      <c r="V76" s="2" t="n"/>
-      <c r="W76" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V76" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W76" s="2" t="n"/>
       <c r="X76" s="2" t="n"/>
       <c r="Y76" s="2" t="inlineStr">
         <is>
@@ -5131,12 +5131,12 @@
         </is>
       </c>
       <c r="U77" s="2" t="n"/>
-      <c r="V77" s="2" t="n"/>
-      <c r="W77" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V77" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W77" s="2" t="n"/>
       <c r="X77" s="2" t="n"/>
       <c r="Y77" s="2" t="inlineStr">
         <is>
@@ -5191,12 +5191,12 @@
         </is>
       </c>
       <c r="U78" s="2" t="n"/>
-      <c r="V78" s="2" t="n"/>
-      <c r="W78" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V78" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W78" s="2" t="n"/>
       <c r="X78" s="2" t="n"/>
       <c r="Y78" s="2" t="n"/>
       <c r="Z78" s="2" t="n"/>
@@ -5251,12 +5251,12 @@
         </is>
       </c>
       <c r="U79" s="2" t="n"/>
-      <c r="V79" s="2" t="n"/>
-      <c r="W79" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V79" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W79" s="2" t="n"/>
       <c r="X79" s="2" t="n"/>
       <c r="Y79" s="2" t="inlineStr">
         <is>
@@ -5313,17 +5313,17 @@
       <c r="U80" s="2" t="n"/>
       <c r="V80" s="2" t="inlineStr">
         <is>
-          <t>BG; PS</t>
-        </is>
-      </c>
-      <c r="W80" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W80" s="2" t="n"/>
       <c r="X80" s="2" t="n"/>
       <c r="Y80" s="2" t="n"/>
-      <c r="Z80" s="2" t="n"/>
+      <c r="Z80" s="2" t="inlineStr">
+        <is>
+          <t>BG; PS</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5367,12 +5367,12 @@
         </is>
       </c>
       <c r="U81" s="2" t="n"/>
-      <c r="V81" s="2" t="n"/>
-      <c r="W81" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V81" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W81" s="2" t="n"/>
       <c r="X81" s="2" t="n"/>
       <c r="Y81" s="2" t="n"/>
       <c r="Z81" s="2" t="n"/>
@@ -5410,12 +5410,12 @@
       </c>
       <c r="V82" t="inlineStr">
         <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
           <t>RW</t>
-        </is>
-      </c>
-      <c r="W82" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
@@ -5465,12 +5465,12 @@
         </is>
       </c>
       <c r="U83" s="2" t="n"/>
-      <c r="V83" s="2" t="n"/>
-      <c r="W83" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V83" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W83" s="2" t="n"/>
       <c r="X83" s="2" t="n"/>
       <c r="Y83" s="2" t="n"/>
       <c r="Z83" s="2" t="n"/>
@@ -5525,12 +5525,12 @@
         </is>
       </c>
       <c r="U84" s="2" t="n"/>
-      <c r="V84" s="2" t="n"/>
-      <c r="W84" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V84" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W84" s="2" t="n"/>
       <c r="X84" s="2" t="n"/>
       <c r="Y84" s="2" t="inlineStr">
         <is>
@@ -5585,12 +5585,12 @@
         </is>
       </c>
       <c r="U85" s="2" t="n"/>
-      <c r="V85" s="2" t="n"/>
-      <c r="W85" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V85" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W85" s="2" t="n"/>
       <c r="X85" s="2" t="n"/>
       <c r="Y85" s="2" t="n"/>
       <c r="Z85" s="2" t="n"/>
@@ -5641,12 +5641,12 @@
         </is>
       </c>
       <c r="U86" s="2" t="n"/>
-      <c r="V86" s="2" t="n"/>
-      <c r="W86" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V86" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W86" s="2" t="n"/>
       <c r="X86" s="2" t="n"/>
       <c r="Y86" s="2" t="n"/>
       <c r="Z86" s="2" t="n"/>
@@ -5693,12 +5693,12 @@
         </is>
       </c>
       <c r="U87" s="2" t="n"/>
-      <c r="V87" s="2" t="n"/>
-      <c r="W87" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V87" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W87" s="2" t="n"/>
       <c r="X87" s="2" t="n"/>
       <c r="Y87" s="2" t="n"/>
       <c r="Z87" s="2" t="n"/>
@@ -5731,12 +5731,12 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
           <t>AW</t>
-        </is>
-      </c>
-      <c r="W88" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
@@ -5788,17 +5788,17 @@
       <c r="U89" s="2" t="n"/>
       <c r="V89" s="2" t="inlineStr">
         <is>
-          <t>BG</t>
-        </is>
-      </c>
-      <c r="W89" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W89" s="2" t="n"/>
       <c r="X89" s="2" t="n"/>
       <c r="Y89" s="2" t="n"/>
-      <c r="Z89" s="2" t="n"/>
+      <c r="Z89" s="2" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5842,12 +5842,12 @@
         </is>
       </c>
       <c r="U90" s="2" t="n"/>
-      <c r="V90" s="2" t="n"/>
-      <c r="W90" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V90" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W90" s="2" t="n"/>
       <c r="X90" s="2" t="n"/>
       <c r="Y90" s="2" t="n"/>
       <c r="Z90" s="2" t="n"/>
@@ -5902,12 +5902,12 @@
         </is>
       </c>
       <c r="U91" s="2" t="n"/>
-      <c r="V91" s="2" t="n"/>
-      <c r="W91" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V91" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W91" s="2" t="n"/>
       <c r="X91" s="2" t="n"/>
       <c r="Y91" s="2" t="inlineStr">
         <is>
@@ -5958,12 +5958,12 @@
         </is>
       </c>
       <c r="U92" s="2" t="n"/>
-      <c r="V92" s="2" t="n"/>
-      <c r="W92" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V92" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W92" s="2" t="n"/>
       <c r="X92" s="2" t="n"/>
       <c r="Y92" s="2" t="n"/>
       <c r="Z92" s="2" t="n"/>
@@ -6018,12 +6018,12 @@
         </is>
       </c>
       <c r="U93" s="2" t="n"/>
-      <c r="V93" s="2" t="n"/>
-      <c r="W93" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V93" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W93" s="2" t="n"/>
       <c r="X93" s="2" t="n"/>
       <c r="Y93" s="2" t="inlineStr">
         <is>
@@ -6082,12 +6082,12 @@
         </is>
       </c>
       <c r="U94" s="2" t="n"/>
-      <c r="V94" s="2" t="n"/>
-      <c r="W94" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V94" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W94" s="2" t="n"/>
       <c r="X94" s="2" t="n"/>
       <c r="Y94" s="2" t="inlineStr">
         <is>
@@ -6146,12 +6146,12 @@
         </is>
       </c>
       <c r="U95" s="2" t="n"/>
-      <c r="V95" s="2" t="n"/>
-      <c r="W95" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V95" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W95" s="2" t="n"/>
       <c r="X95" s="2" t="n"/>
       <c r="Y95" s="2" t="inlineStr">
         <is>
@@ -6210,12 +6210,12 @@
         </is>
       </c>
       <c r="U96" s="2" t="n"/>
-      <c r="V96" s="2" t="n"/>
-      <c r="W96" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V96" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W96" s="2" t="n"/>
       <c r="X96" s="2" t="n"/>
       <c r="Y96" s="2" t="inlineStr">
         <is>
@@ -6274,12 +6274,12 @@
         </is>
       </c>
       <c r="U97" s="2" t="n"/>
-      <c r="V97" s="2" t="n"/>
-      <c r="W97" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V97" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W97" s="2" t="n"/>
       <c r="X97" s="2" t="n"/>
       <c r="Y97" s="2" t="inlineStr">
         <is>
@@ -6334,12 +6334,12 @@
         </is>
       </c>
       <c r="U98" s="2" t="n"/>
-      <c r="V98" s="2" t="n"/>
-      <c r="W98" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V98" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W98" s="2" t="n"/>
       <c r="X98" s="2" t="n"/>
       <c r="Y98" s="2" t="n"/>
       <c r="Z98" s="2" t="n"/>
@@ -6390,12 +6390,12 @@
         </is>
       </c>
       <c r="U99" s="2" t="n"/>
-      <c r="V99" s="2" t="n"/>
-      <c r="W99" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V99" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W99" s="2" t="n"/>
       <c r="X99" s="2" t="n"/>
       <c r="Y99" s="2" t="inlineStr">
         <is>
@@ -6450,12 +6450,12 @@
         </is>
       </c>
       <c r="U100" s="2" t="n"/>
-      <c r="V100" s="2" t="n"/>
-      <c r="W100" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V100" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W100" s="2" t="n"/>
       <c r="X100" s="2" t="n"/>
       <c r="Y100" s="2" t="inlineStr">
         <is>
@@ -6514,12 +6514,12 @@
         </is>
       </c>
       <c r="U101" s="2" t="n"/>
-      <c r="V101" s="2" t="n"/>
-      <c r="W101" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V101" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W101" s="2" t="n"/>
       <c r="X101" s="2" t="n"/>
       <c r="Y101" s="2" t="inlineStr">
         <is>
@@ -6570,12 +6570,12 @@
         </is>
       </c>
       <c r="U102" s="2" t="n"/>
-      <c r="V102" s="2" t="n"/>
-      <c r="W102" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V102" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W102" s="2" t="n"/>
       <c r="X102" s="2" t="n"/>
       <c r="Y102" s="2" t="n"/>
       <c r="Z102" s="2" t="n"/>
@@ -6630,12 +6630,12 @@
         </is>
       </c>
       <c r="U103" s="2" t="n"/>
-      <c r="V103" s="2" t="n"/>
-      <c r="W103" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V103" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W103" s="2" t="n"/>
       <c r="X103" s="2" t="n"/>
       <c r="Y103" s="2" t="inlineStr">
         <is>
@@ -6686,12 +6686,12 @@
         </is>
       </c>
       <c r="U104" s="2" t="n"/>
-      <c r="V104" s="2" t="n"/>
-      <c r="W104" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V104" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W104" s="2" t="n"/>
       <c r="X104" s="2" t="n"/>
       <c r="Y104" s="2" t="n"/>
       <c r="Z104" s="2" t="n"/>
@@ -6746,12 +6746,12 @@
         </is>
       </c>
       <c r="U105" s="2" t="n"/>
-      <c r="V105" s="2" t="n"/>
-      <c r="W105" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V105" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W105" s="2" t="n"/>
       <c r="X105" s="2" t="n"/>
       <c r="Y105" s="2" t="inlineStr">
         <is>
@@ -6806,12 +6806,12 @@
         </is>
       </c>
       <c r="U106" s="2" t="n"/>
-      <c r="V106" s="2" t="n"/>
-      <c r="W106" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V106" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W106" s="2" t="n"/>
       <c r="X106" s="2" t="n"/>
       <c r="Y106" s="2" t="n"/>
       <c r="Z106" s="2" t="n"/>
@@ -6866,12 +6866,12 @@
         </is>
       </c>
       <c r="U107" s="2" t="n"/>
-      <c r="V107" s="2" t="n"/>
-      <c r="W107" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V107" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W107" s="2" t="n"/>
       <c r="X107" s="2" t="n"/>
       <c r="Y107" s="2" t="inlineStr">
         <is>
@@ -6926,12 +6926,12 @@
         </is>
       </c>
       <c r="U108" s="2" t="n"/>
-      <c r="V108" s="2" t="n"/>
-      <c r="W108" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V108" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W108" s="2" t="n"/>
       <c r="X108" s="2" t="n"/>
       <c r="Y108" s="2" t="n"/>
       <c r="Z108" s="2" t="n"/>
@@ -6982,12 +6982,12 @@
         </is>
       </c>
       <c r="U109" s="2" t="n"/>
-      <c r="V109" s="2" t="n"/>
-      <c r="W109" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V109" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W109" s="2" t="n"/>
       <c r="X109" s="2" t="n"/>
       <c r="Y109" s="2" t="n"/>
       <c r="Z109" s="2" t="n"/>
@@ -7042,12 +7042,12 @@
         </is>
       </c>
       <c r="U110" s="2" t="n"/>
-      <c r="V110" s="2" t="n"/>
-      <c r="W110" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V110" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W110" s="2" t="n"/>
       <c r="X110" s="2" t="n"/>
       <c r="Y110" s="2" t="inlineStr">
         <is>
@@ -7098,12 +7098,12 @@
         </is>
       </c>
       <c r="U111" s="2" t="n"/>
-      <c r="V111" s="2" t="n"/>
-      <c r="W111" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V111" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W111" s="2" t="n"/>
       <c r="X111" s="2" t="n"/>
       <c r="Y111" s="2" t="n"/>
       <c r="Z111" s="2" t="n"/>
@@ -7158,12 +7158,12 @@
         </is>
       </c>
       <c r="U112" s="2" t="n"/>
-      <c r="V112" s="2" t="n"/>
-      <c r="W112" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V112" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W112" s="2" t="n"/>
       <c r="X112" s="2" t="n"/>
       <c r="Y112" s="2" t="inlineStr">
         <is>
@@ -7222,12 +7222,12 @@
         </is>
       </c>
       <c r="U113" s="2" t="n"/>
-      <c r="V113" s="2" t="n"/>
-      <c r="W113" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V113" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W113" s="2" t="n"/>
       <c r="X113" s="2" t="n"/>
       <c r="Y113" s="2" t="inlineStr">
         <is>
@@ -7282,12 +7282,12 @@
         </is>
       </c>
       <c r="U114" s="2" t="n"/>
-      <c r="V114" s="2" t="n"/>
-      <c r="W114" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V114" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W114" s="2" t="n"/>
       <c r="X114" s="2" t="n"/>
       <c r="Y114" s="2" t="inlineStr">
         <is>
@@ -7342,12 +7342,12 @@
         </is>
       </c>
       <c r="U115" s="2" t="n"/>
-      <c r="V115" s="2" t="n"/>
-      <c r="W115" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V115" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W115" s="2" t="n"/>
       <c r="X115" s="2" t="n"/>
       <c r="Y115" s="2" t="n"/>
       <c r="Z115" s="2" t="n"/>
@@ -7402,12 +7402,12 @@
         </is>
       </c>
       <c r="U116" s="2" t="n"/>
-      <c r="V116" s="2" t="n"/>
-      <c r="W116" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V116" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W116" s="2" t="n"/>
       <c r="X116" s="2" t="n"/>
       <c r="Y116" s="2" t="inlineStr">
         <is>
@@ -7466,12 +7466,12 @@
         </is>
       </c>
       <c r="U117" s="2" t="n"/>
-      <c r="V117" s="2" t="n"/>
-      <c r="W117" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V117" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W117" s="2" t="n"/>
       <c r="X117" s="2" t="n"/>
       <c r="Y117" s="2" t="inlineStr">
         <is>
@@ -7530,12 +7530,12 @@
         </is>
       </c>
       <c r="U118" s="2" t="n"/>
-      <c r="V118" s="2" t="n"/>
-      <c r="W118" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V118" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W118" s="2" t="n"/>
       <c r="X118" s="2" t="n"/>
       <c r="Y118" s="2" t="inlineStr">
         <is>
@@ -7594,12 +7594,12 @@
         </is>
       </c>
       <c r="U119" s="2" t="n"/>
-      <c r="V119" s="2" t="n"/>
-      <c r="W119" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V119" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W119" s="2" t="n"/>
       <c r="X119" s="2" t="n"/>
       <c r="Y119" s="2" t="inlineStr">
         <is>
@@ -7654,12 +7654,12 @@
         </is>
       </c>
       <c r="U120" s="2" t="n"/>
-      <c r="V120" s="2" t="n"/>
-      <c r="W120" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V120" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W120" s="2" t="n"/>
       <c r="X120" s="2" t="n"/>
       <c r="Y120" s="2" t="n"/>
       <c r="Z120" s="2" t="n"/>
@@ -7706,12 +7706,12 @@
         </is>
       </c>
       <c r="U121" s="2" t="n"/>
-      <c r="V121" s="2" t="n"/>
-      <c r="W121" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V121" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W121" s="2" t="n"/>
       <c r="X121" s="2" t="n"/>
       <c r="Y121" s="2" t="n"/>
       <c r="Z121" s="2" t="n"/>
@@ -7758,12 +7758,12 @@
         </is>
       </c>
       <c r="U122" s="2" t="n"/>
-      <c r="V122" s="2" t="n"/>
-      <c r="W122" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V122" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W122" s="2" t="n"/>
       <c r="X122" s="2" t="n"/>
       <c r="Y122" s="2" t="n"/>
       <c r="Z122" s="2" t="n"/>
@@ -7810,12 +7810,12 @@
         </is>
       </c>
       <c r="U123" s="2" t="n"/>
-      <c r="V123" s="2" t="n"/>
-      <c r="W123" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V123" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W123" s="2" t="n"/>
       <c r="X123" s="2" t="n"/>
       <c r="Y123" s="2" t="n"/>
       <c r="Z123" s="2" t="n"/>
@@ -7870,12 +7870,12 @@
         </is>
       </c>
       <c r="U124" s="2" t="n"/>
-      <c r="V124" s="2" t="n"/>
-      <c r="W124" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V124" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W124" s="2" t="n"/>
       <c r="X124" s="2" t="n"/>
       <c r="Y124" s="2" t="inlineStr">
         <is>
@@ -7934,12 +7934,12 @@
         </is>
       </c>
       <c r="U125" s="2" t="n"/>
-      <c r="V125" s="2" t="n"/>
-      <c r="W125" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V125" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W125" s="2" t="n"/>
       <c r="X125" s="2" t="n"/>
       <c r="Y125" s="2" t="inlineStr">
         <is>
@@ -7998,12 +7998,12 @@
         </is>
       </c>
       <c r="U126" s="2" t="n"/>
-      <c r="V126" s="2" t="n"/>
-      <c r="W126" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V126" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W126" s="2" t="n"/>
       <c r="X126" s="2" t="n"/>
       <c r="Y126" s="2" t="inlineStr">
         <is>
@@ -8062,12 +8062,12 @@
         </is>
       </c>
       <c r="U127" s="2" t="n"/>
-      <c r="V127" s="2" t="n"/>
-      <c r="W127" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V127" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W127" s="2" t="n"/>
       <c r="X127" s="2" t="n"/>
       <c r="Y127" s="2" t="inlineStr">
         <is>
@@ -8122,12 +8122,12 @@
         </is>
       </c>
       <c r="U128" s="2" t="n"/>
-      <c r="V128" s="2" t="n"/>
-      <c r="W128" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V128" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W128" s="2" t="n"/>
       <c r="X128" s="2" t="n"/>
       <c r="Y128" s="2" t="n"/>
       <c r="Z128" s="2" t="n"/>
@@ -8176,17 +8176,17 @@
       <c r="U129" s="2" t="n"/>
       <c r="V129" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W129" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W129" s="2" t="n"/>
       <c r="X129" s="2" t="n"/>
       <c r="Y129" s="2" t="n"/>
-      <c r="Z129" s="2" t="n"/>
+      <c r="Z129" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8238,12 +8238,12 @@
         </is>
       </c>
       <c r="U130" s="2" t="n"/>
-      <c r="V130" s="2" t="n"/>
-      <c r="W130" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V130" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W130" s="2" t="n"/>
       <c r="X130" s="2" t="n"/>
       <c r="Y130" s="2" t="n"/>
       <c r="Z130" s="2" t="n"/>
@@ -8294,12 +8294,12 @@
         </is>
       </c>
       <c r="U131" s="2" t="n"/>
-      <c r="V131" s="2" t="n"/>
-      <c r="W131" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V131" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W131" s="2" t="n"/>
       <c r="X131" s="2" t="n"/>
       <c r="Y131" s="2" t="n"/>
       <c r="Z131" s="2" t="n"/>
@@ -8354,12 +8354,12 @@
         </is>
       </c>
       <c r="U132" s="2" t="n"/>
-      <c r="V132" s="2" t="n"/>
-      <c r="W132" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V132" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W132" s="2" t="n"/>
       <c r="X132" s="2" t="n"/>
       <c r="Y132" s="2" t="inlineStr">
         <is>
@@ -8418,12 +8418,12 @@
         </is>
       </c>
       <c r="U133" s="2" t="n"/>
-      <c r="V133" s="2" t="n"/>
-      <c r="W133" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V133" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W133" s="2" t="n"/>
       <c r="X133" s="2" t="n"/>
       <c r="Y133" s="2" t="inlineStr">
         <is>
@@ -8478,12 +8478,12 @@
         </is>
       </c>
       <c r="U134" s="2" t="n"/>
-      <c r="V134" s="2" t="n"/>
-      <c r="W134" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V134" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W134" s="2" t="n"/>
       <c r="X134" s="2" t="n"/>
       <c r="Y134" s="2" t="inlineStr">
         <is>
@@ -8538,12 +8538,12 @@
         </is>
       </c>
       <c r="U135" s="2" t="n"/>
-      <c r="V135" s="2" t="n"/>
-      <c r="W135" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V135" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W135" s="2" t="n"/>
       <c r="X135" s="2" t="n"/>
       <c r="Y135" s="2" t="n"/>
       <c r="Z135" s="2" t="n"/>
@@ -8598,12 +8598,12 @@
         </is>
       </c>
       <c r="U136" s="2" t="n"/>
-      <c r="V136" s="2" t="n"/>
-      <c r="W136" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V136" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W136" s="2" t="n"/>
       <c r="X136" s="2" t="n"/>
       <c r="Y136" s="2" t="inlineStr">
         <is>
@@ -8662,12 +8662,12 @@
         </is>
       </c>
       <c r="U137" s="2" t="n"/>
-      <c r="V137" s="2" t="n"/>
-      <c r="W137" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V137" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W137" s="2" t="n"/>
       <c r="X137" s="2" t="n"/>
       <c r="Y137" s="2" t="inlineStr">
         <is>
@@ -8679,22 +8679,22 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010089</t>
+          <t>BCIO:010087</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>undergraduate student role</t>
+          <t>trainee role</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
+          <t>A student or trainee role that is currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>higher education student role</t>
+          <t>student or trainee role</t>
         </is>
       </c>
       <c r="E138" s="2" t="n"/>
@@ -8709,11 +8709,7 @@
       <c r="N138" s="2" t="n"/>
       <c r="O138" s="2" t="n"/>
       <c r="P138" s="2" t="n"/>
-      <c r="Q138" s="2" t="inlineStr">
-        <is>
-          <t>undergraduate student</t>
-        </is>
-      </c>
+      <c r="Q138" s="2" t="n"/>
       <c r="R138" s="2" t="n"/>
       <c r="S138" s="2" t="n"/>
       <c r="T138" s="2" t="inlineStr">
@@ -8722,12 +8718,12 @@
         </is>
       </c>
       <c r="U138" s="2" t="n"/>
-      <c r="V138" s="2" t="n"/>
-      <c r="W138" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V138" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W138" s="2" t="n"/>
       <c r="X138" s="2" t="n"/>
       <c r="Y138" s="2" t="n"/>
       <c r="Z138" s="2" t="n"/>
@@ -8735,23 +8731,22 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010026</t>
+          <t>BCIO:010089</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">university and higher education teacher
-</t>
+          <t>undergraduate student role</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>A teaching professional that prepares and delivers lectures and conduct tutorials in one or more subjects within a prescribed course of study at a university or other higher educational institution. They conduct research, and prepare scholarly papers and books.</t>
+          <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">teaching professional </t>
+          <t>higher education student role</t>
         </is>
       </c>
       <c r="E139" s="2" t="n"/>
@@ -8768,14 +8763,10 @@
       <c r="P139" s="2" t="n"/>
       <c r="Q139" s="2" t="inlineStr">
         <is>
-          <t>Higher education lecturer, Professor, University lecturer, University tutor</t>
-        </is>
-      </c>
-      <c r="R139" s="2" t="inlineStr">
-        <is>
-          <t>International Standard Classification of Occupations (ISCO)</t>
-        </is>
-      </c>
+          <t>undergraduate student</t>
+        </is>
+      </c>
+      <c r="R139" s="2" t="n"/>
       <c r="S139" s="2" t="n"/>
       <c r="T139" s="2" t="inlineStr">
         <is>
@@ -8783,39 +8774,36 @@
         </is>
       </c>
       <c r="U139" s="2" t="n"/>
-      <c r="V139" s="2" t="n"/>
-      <c r="W139" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V139" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W139" s="2" t="n"/>
       <c r="X139" s="2" t="n"/>
-      <c r="Y139" s="2" t="inlineStr">
-        <is>
-          <t>ISCO: 231</t>
-        </is>
-      </c>
+      <c r="Y139" s="2" t="n"/>
       <c r="Z139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010017</t>
+          <t>BCIO:010026</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">veterinarian </t>
+          <t xml:space="preserve">university and higher education teacher
+</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A health professional that diagnoses, prevents and treats diseases, injuries and dysfunctions of animals. </t>
+          <t>A teaching professional that prepares and delivers lectures and conduct tutorials in one or more subjects within a prescribed course of study at a university or other higher educational institution. They conduct research, and prepare scholarly papers and books.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">health professional </t>
+          <t xml:space="preserve">teaching professional </t>
         </is>
       </c>
       <c r="E140" s="2" t="n"/>
@@ -8832,7 +8820,7 @@
       <c r="P140" s="2" t="n"/>
       <c r="Q140" s="2" t="inlineStr">
         <is>
-          <t>Animal pathologist, Veterinarian, Veterinary epidemiologist, Veterinary intern, Veterinary surgeon</t>
+          <t>Higher education lecturer, Professor, University lecturer, University tutor</t>
         </is>
       </c>
       <c r="R140" s="2" t="inlineStr">
@@ -8847,16 +8835,16 @@
         </is>
       </c>
       <c r="U140" s="2" t="n"/>
-      <c r="V140" s="2" t="n"/>
-      <c r="W140" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V140" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W140" s="2" t="n"/>
       <c r="X140" s="2" t="n"/>
       <c r="Y140" s="2" t="inlineStr">
         <is>
-          <t>ISCO: 225</t>
+          <t>ISCO: 231</t>
         </is>
       </c>
       <c r="Z140" s="2" t="n"/>
@@ -8864,22 +8852,22 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010027</t>
+          <t>BCIO:010017</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>vocational education teacher</t>
+          <t xml:space="preserve">veterinarian </t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A teaching professional that teaches or instructs vocational or occupational subjects in adult and further education institutions and to senior students in secondary schools and colleges. </t>
+          <t xml:space="preserve">A health professional that diagnoses, prevents and treats diseases, injuries and dysfunctions of animals. </t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">teaching professional </t>
+          <t xml:space="preserve">health professional </t>
         </is>
       </c>
       <c r="E141" s="2" t="n"/>
@@ -8896,7 +8884,7 @@
       <c r="P141" s="2" t="n"/>
       <c r="Q141" s="2" t="inlineStr">
         <is>
-          <t>Automotive technology instructor, Cosmetology instructor, Vocational education teacher</t>
+          <t>Animal pathologist, Veterinarian, Veterinary epidemiologist, Veterinary intern, Veterinary surgeon</t>
         </is>
       </c>
       <c r="R141" s="2" t="inlineStr">
@@ -8911,16 +8899,16 @@
         </is>
       </c>
       <c r="U141" s="2" t="n"/>
-      <c r="V141" s="2" t="n"/>
-      <c r="W141" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V141" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W141" s="2" t="n"/>
       <c r="X141" s="2" t="n"/>
       <c r="Y141" s="2" t="inlineStr">
         <is>
-          <t>ISCO: 232</t>
+          <t>ISCO: 225</t>
         </is>
       </c>
       <c r="Z141" s="2" t="n"/>
@@ -8928,22 +8916,22 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010087</t>
+          <t>BCIO:010027</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>vocational training student or trainee role</t>
+          <t>vocational education teacher</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>A student or trainee role that is currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
+          <t xml:space="preserve">A teaching professional that teaches or instructs vocational or occupational subjects in adult and further education institutions and to senior students in secondary schools and colleges. </t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>student or trainee role</t>
+          <t xml:space="preserve">teaching professional </t>
         </is>
       </c>
       <c r="E142" s="2" t="n"/>
@@ -8958,8 +8946,16 @@
       <c r="N142" s="2" t="n"/>
       <c r="O142" s="2" t="n"/>
       <c r="P142" s="2" t="n"/>
-      <c r="Q142" s="2" t="n"/>
-      <c r="R142" s="2" t="n"/>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>Automotive technology instructor, Cosmetology instructor, Vocational education teacher</t>
+        </is>
+      </c>
+      <c r="R142" s="2" t="inlineStr">
+        <is>
+          <t>International Standard Classification of Occupations (ISCO)</t>
+        </is>
+      </c>
       <c r="S142" s="2" t="n"/>
       <c r="T142" s="2" t="inlineStr">
         <is>
@@ -8967,14 +8963,18 @@
         </is>
       </c>
       <c r="U142" s="2" t="n"/>
-      <c r="V142" s="2" t="n"/>
-      <c r="W142" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V142" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W142" s="2" t="n"/>
       <c r="X142" s="2" t="n"/>
-      <c r="Y142" s="2" t="n"/>
+      <c r="Y142" s="2" t="inlineStr">
+        <is>
+          <t>ISCO: 232</t>
+        </is>
+      </c>
       <c r="Z142" s="2" t="n"/>
     </row>
     <row r="143">
@@ -9027,12 +9027,12 @@
         </is>
       </c>
       <c r="U143" s="2" t="n"/>
-      <c r="V143" s="2" t="n"/>
-      <c r="W143" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V143" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W143" s="2" t="n"/>
       <c r="X143" s="2" t="n"/>
       <c r="Y143" s="2" t="n"/>
       <c r="Z143" s="2" t="n"/>

</xml_diff>

<commit_message>
Update behaviour change intervention study investigator role in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +40,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007fffd4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,11 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1350,48 +1344,48 @@
       <c r="Z14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>BCIO:030000</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>behaviour change intervention study investigator role</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>researcher</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr"/>
-      <c r="O15" s="3" t="inlineStr"/>
-      <c r="P15" s="3" t="inlineStr"/>
-      <c r="Q15" s="3" t="inlineStr"/>
-      <c r="R15" s="3" t="inlineStr"/>
-      <c r="S15" s="3" t="inlineStr"/>
-      <c r="T15" s="3" t="inlineStr"/>
-      <c r="U15" s="3" t="inlineStr"/>
-      <c r="V15" s="3" t="inlineStr"/>
-      <c r="W15" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="X15" s="3" t="inlineStr"/>
-      <c r="Y15" s="3" t="inlineStr"/>
-      <c r="Z15" s="3" t="inlineStr"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2" t="n"/>
+      <c r="O15" s="2" t="n"/>
+      <c r="P15" s="2" t="n"/>
+      <c r="Q15" s="2" t="n"/>
+      <c r="R15" s="2" t="n"/>
+      <c r="S15" s="2" t="n"/>
+      <c r="T15" s="2" t="n"/>
+      <c r="U15" s="2" t="n"/>
+      <c r="V15" s="2" t="n"/>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="n"/>
+      <c r="Y15" s="2" t="n"/>
+      <c r="Z15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 2 terms in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -1361,7 +1361,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>researcher</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -6936,12 +6936,12 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>researcher</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study</t>
+          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 3 terms in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +40,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007fffd4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,10 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,27 +541,27 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>To be reviewed by</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer query</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Definition_ID</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Curator</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>To be reviewed by</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_ID</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Reviewer query</t>
         </is>
       </c>
     </row>
@@ -567,17 +573,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>acquired knowledge or skill</t>
+          <t>acquired expertise</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>A knowledge or skill that is additional knowledge or skills supplied to the source to allow them to deliver the behaviour change intervention, including educational level and qualifications.</t>
+          <t>An expertise of person source that is additional knowledge or skills supplied to the source to allow them to deliver the intervention, including educational level and qualifications.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>knowledge or skill</t>
+          <t>expertise of person source</t>
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
@@ -601,12 +607,12 @@
         </is>
       </c>
       <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="n"/>
       <c r="Z2" s="2" t="n"/>
@@ -657,12 +663,12 @@
         </is>
       </c>
       <c r="U3" s="2" t="n"/>
-      <c r="V3" s="2" t="n"/>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="n"/>
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="n"/>
       <c r="Z3" s="2" t="n"/>
@@ -709,12 +715,12 @@
         </is>
       </c>
       <c r="U4" s="2" t="n"/>
-      <c r="V4" s="2" t="n"/>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="n"/>
       <c r="X4" s="2" t="n"/>
       <c r="Y4" s="2" t="n"/>
       <c r="Z4" s="2" t="n"/>
@@ -769,12 +775,12 @@
         </is>
       </c>
       <c r="U5" s="2" t="n"/>
-      <c r="V5" s="2" t="n"/>
-      <c r="W5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="n"/>
       <c r="X5" s="2" t="n"/>
       <c r="Y5" s="2" t="inlineStr">
         <is>
@@ -833,12 +839,12 @@
         </is>
       </c>
       <c r="U6" s="2" t="n"/>
-      <c r="V6" s="2" t="n"/>
-      <c r="W6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="n"/>
       <c r="X6" s="2" t="n"/>
       <c r="Y6" s="2" t="n"/>
       <c r="Z6" s="2" t="n"/>
@@ -893,12 +899,12 @@
         </is>
       </c>
       <c r="U7" s="2" t="n"/>
-      <c r="V7" s="2" t="n"/>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="n"/>
       <c r="X7" s="2" t="n"/>
       <c r="Y7" s="2" t="inlineStr">
         <is>
@@ -957,12 +963,12 @@
         </is>
       </c>
       <c r="U8" s="2" t="n"/>
-      <c r="V8" s="2" t="n"/>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="n"/>
       <c r="X8" s="2" t="n"/>
       <c r="Y8" s="2" t="inlineStr">
         <is>
@@ -1021,12 +1027,12 @@
         </is>
       </c>
       <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="n"/>
-      <c r="W9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="n"/>
       <c r="X9" s="2" t="n"/>
       <c r="Y9" s="2" t="inlineStr">
         <is>
@@ -1081,12 +1087,12 @@
         </is>
       </c>
       <c r="U10" s="2" t="n"/>
-      <c r="V10" s="2" t="n"/>
-      <c r="W10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="n"/>
       <c r="X10" s="2" t="n"/>
       <c r="Y10" s="2" t="inlineStr">
         <is>
@@ -1145,12 +1151,12 @@
         </is>
       </c>
       <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="n"/>
-      <c r="W11" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="n"/>
       <c r="X11" s="2" t="n"/>
       <c r="Y11" s="2" t="inlineStr">
         <is>
@@ -1209,12 +1215,12 @@
         </is>
       </c>
       <c r="U12" s="2" t="n"/>
-      <c r="V12" s="2" t="n"/>
-      <c r="W12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="n"/>
       <c r="X12" s="2" t="n"/>
       <c r="Y12" s="2" t="inlineStr">
         <is>
@@ -1273,12 +1279,12 @@
         </is>
       </c>
       <c r="U13" s="2" t="n"/>
-      <c r="V13" s="2" t="n"/>
-      <c r="W13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="n"/>
       <c r="X13" s="2" t="n"/>
       <c r="Y13" s="2" t="inlineStr">
         <is>
@@ -1331,17 +1337,17 @@
       <c r="U14" s="2" t="n"/>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="W14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="n"/>
       <c r="X14" s="2" t="n"/>
       <c r="Y14" s="2" t="n"/>
-      <c r="Z14" s="2" t="n"/>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1381,12 +1387,12 @@
       <c r="S15" s="2" t="n"/>
       <c r="T15" s="2" t="n"/>
       <c r="U15" s="2" t="n"/>
-      <c r="V15" s="2" t="n"/>
-      <c r="W15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="n"/>
       <c r="X15" s="2" t="n"/>
       <c r="Y15" s="2" t="n"/>
       <c r="Z15" s="2" t="n"/>
@@ -1441,12 +1447,12 @@
         </is>
       </c>
       <c r="U16" s="2" t="n"/>
-      <c r="V16" s="2" t="n"/>
-      <c r="W16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="n"/>
       <c r="X16" s="2" t="n"/>
       <c r="Y16" s="2" t="inlineStr">
         <is>
@@ -1501,12 +1507,12 @@
         </is>
       </c>
       <c r="U17" s="2" t="n"/>
-      <c r="V17" s="2" t="n"/>
-      <c r="W17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="n"/>
       <c r="X17" s="2" t="n"/>
       <c r="Y17" s="2" t="n"/>
       <c r="Z17" s="2" t="n"/>
@@ -1561,12 +1567,12 @@
         </is>
       </c>
       <c r="U18" s="2" t="n"/>
-      <c r="V18" s="2" t="n"/>
-      <c r="W18" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="n"/>
       <c r="X18" s="2" t="n"/>
       <c r="Y18" s="2" t="inlineStr">
         <is>
@@ -1621,12 +1627,12 @@
         </is>
       </c>
       <c r="U19" s="2" t="n"/>
-      <c r="V19" s="2" t="n"/>
-      <c r="W19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="n"/>
       <c r="X19" s="2" t="n"/>
       <c r="Y19" s="2" t="n"/>
       <c r="Z19" s="2" t="n"/>
@@ -1681,12 +1687,12 @@
         </is>
       </c>
       <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="n"/>
-      <c r="W20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="n"/>
       <c r="X20" s="2" t="n"/>
       <c r="Y20" s="2" t="inlineStr">
         <is>
@@ -1737,12 +1743,12 @@
         </is>
       </c>
       <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="n"/>
-      <c r="W21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="n"/>
       <c r="X21" s="2" t="n"/>
       <c r="Y21" s="2" t="n"/>
       <c r="Z21" s="2" t="n"/>
@@ -1797,12 +1803,12 @@
         </is>
       </c>
       <c r="U22" s="2" t="n"/>
-      <c r="V22" s="2" t="n"/>
-      <c r="W22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="n"/>
       <c r="X22" s="2" t="n"/>
       <c r="Y22" s="2" t="inlineStr">
         <is>
@@ -1861,12 +1867,12 @@
         </is>
       </c>
       <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
-      <c r="W23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="n"/>
       <c r="X23" s="2" t="n"/>
       <c r="Y23" s="2" t="inlineStr">
         <is>
@@ -1925,12 +1931,12 @@
         </is>
       </c>
       <c r="U24" s="2" t="n"/>
-      <c r="V24" s="2" t="n"/>
-      <c r="W24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="n"/>
       <c r="X24" s="2" t="n"/>
       <c r="Y24" s="2" t="inlineStr">
         <is>
@@ -1989,12 +1995,12 @@
         </is>
       </c>
       <c r="U25" s="2" t="n"/>
-      <c r="V25" s="2" t="n"/>
-      <c r="W25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="n"/>
       <c r="X25" s="2" t="n"/>
       <c r="Y25" s="2" t="inlineStr">
         <is>
@@ -2053,12 +2059,12 @@
         </is>
       </c>
       <c r="U26" s="2" t="n"/>
-      <c r="V26" s="2" t="n"/>
-      <c r="W26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="n"/>
       <c r="X26" s="2" t="n"/>
       <c r="Y26" s="2" t="inlineStr">
         <is>
@@ -2117,12 +2123,12 @@
         </is>
       </c>
       <c r="U27" s="2" t="n"/>
-      <c r="V27" s="2" t="n"/>
-      <c r="W27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="n"/>
       <c r="X27" s="2" t="n"/>
       <c r="Y27" s="2" t="inlineStr">
         <is>
@@ -2179,17 +2185,17 @@
       <c r="U28" s="2" t="n"/>
       <c r="V28" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="n"/>
       <c r="X28" s="2" t="n"/>
       <c r="Y28" s="2" t="n"/>
-      <c r="Z28" s="2" t="n"/>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2241,12 +2247,12 @@
         </is>
       </c>
       <c r="U29" s="2" t="n"/>
-      <c r="V29" s="2" t="n"/>
-      <c r="W29" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="n"/>
       <c r="X29" s="2" t="n"/>
       <c r="Y29" s="2" t="n"/>
       <c r="Z29" s="2" t="n"/>
@@ -2297,12 +2303,12 @@
         </is>
       </c>
       <c r="U30" s="2" t="n"/>
-      <c r="V30" s="2" t="n"/>
-      <c r="W30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="n"/>
       <c r="X30" s="2" t="n"/>
       <c r="Y30" s="2" t="n"/>
       <c r="Z30" s="2" t="n"/>
@@ -2357,12 +2363,12 @@
         </is>
       </c>
       <c r="U31" s="2" t="n"/>
-      <c r="V31" s="2" t="n"/>
-      <c r="W31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="n"/>
       <c r="X31" s="2" t="n"/>
       <c r="Y31" s="2" t="inlineStr">
         <is>
@@ -2421,12 +2427,12 @@
         </is>
       </c>
       <c r="U32" s="2" t="n"/>
-      <c r="V32" s="2" t="n"/>
-      <c r="W32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="n"/>
       <c r="X32" s="2" t="n"/>
       <c r="Y32" s="2" t="inlineStr">
         <is>
@@ -2477,12 +2483,12 @@
         </is>
       </c>
       <c r="U33" s="2" t="n"/>
-      <c r="V33" s="2" t="n"/>
-      <c r="W33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="2" t="n"/>
       <c r="Z33" s="2" t="n"/>
@@ -2529,12 +2535,12 @@
         </is>
       </c>
       <c r="U34" s="2" t="n"/>
-      <c r="V34" s="2" t="n"/>
-      <c r="W34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="n"/>
       <c r="X34" s="2" t="n"/>
       <c r="Y34" s="2" t="n"/>
       <c r="Z34" s="2" t="n"/>
@@ -2589,12 +2595,12 @@
         </is>
       </c>
       <c r="U35" s="2" t="n"/>
-      <c r="V35" s="2" t="n"/>
-      <c r="W35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="n"/>
       <c r="X35" s="2" t="n"/>
       <c r="Y35" s="2" t="inlineStr">
         <is>
@@ -2655,12 +2661,12 @@
         </is>
       </c>
       <c r="U36" s="2" t="n"/>
-      <c r="V36" s="2" t="n"/>
-      <c r="W36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="n"/>
       <c r="X36" s="2" t="n"/>
       <c r="Y36" s="2" t="inlineStr">
         <is>
@@ -2715,12 +2721,12 @@
         </is>
       </c>
       <c r="U37" s="2" t="n"/>
-      <c r="V37" s="2" t="n"/>
-      <c r="W37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="n"/>
       <c r="X37" s="2" t="n"/>
       <c r="Y37" s="2" t="n"/>
       <c r="Z37" s="2" t="n"/>
@@ -2775,12 +2781,12 @@
         </is>
       </c>
       <c r="U38" s="2" t="n"/>
-      <c r="V38" s="2" t="n"/>
-      <c r="W38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="n"/>
       <c r="X38" s="2" t="n"/>
       <c r="Y38" s="2" t="n"/>
       <c r="Z38" s="2" t="n"/>
@@ -2831,12 +2837,12 @@
         </is>
       </c>
       <c r="U39" s="2" t="n"/>
-      <c r="V39" s="2" t="n"/>
-      <c r="W39" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="n"/>
       <c r="X39" s="2" t="n"/>
       <c r="Y39" s="2" t="n"/>
       <c r="Z39" s="2" t="n"/>
@@ -2885,17 +2891,17 @@
       <c r="U40" s="2" t="n"/>
       <c r="V40" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W40" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W40" s="2" t="n"/>
       <c r="X40" s="2" t="n"/>
       <c r="Y40" s="2" t="n"/>
-      <c r="Z40" s="2" t="n"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2945,17 +2951,17 @@
       <c r="U41" s="2" t="n"/>
       <c r="V41" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W41" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W41" s="2" t="n"/>
       <c r="X41" s="2" t="n"/>
       <c r="Y41" s="2" t="n"/>
-      <c r="Z41" s="2" t="n"/>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3007,12 +3013,12 @@
         </is>
       </c>
       <c r="U42" s="2" t="n"/>
-      <c r="V42" s="2" t="n"/>
-      <c r="W42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="n"/>
       <c r="X42" s="2" t="n"/>
       <c r="Y42" s="2" t="inlineStr">
         <is>
@@ -3063,12 +3069,12 @@
         </is>
       </c>
       <c r="U43" s="2" t="n"/>
-      <c r="V43" s="2" t="n"/>
-      <c r="W43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W43" s="2" t="n"/>
       <c r="X43" s="2" t="n"/>
       <c r="Y43" s="2" t="n"/>
       <c r="Z43" s="2" t="n"/>
@@ -3117,17 +3123,17 @@
       <c r="U44" s="2" t="n"/>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W44" s="2" t="n"/>
       <c r="X44" s="2" t="n"/>
       <c r="Y44" s="2" t="n"/>
-      <c r="Z44" s="2" t="n"/>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3175,12 +3181,12 @@
         </is>
       </c>
       <c r="U45" s="2" t="n"/>
-      <c r="V45" s="2" t="n"/>
-      <c r="W45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W45" s="2" t="n"/>
       <c r="X45" s="2" t="n"/>
       <c r="Y45" s="2" t="n"/>
       <c r="Z45" s="2" t="n"/>
@@ -3235,12 +3241,12 @@
         </is>
       </c>
       <c r="U46" s="2" t="n"/>
-      <c r="V46" s="2" t="n"/>
-      <c r="W46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V46" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W46" s="2" t="n"/>
       <c r="X46" s="2" t="n"/>
       <c r="Y46" s="2" t="inlineStr">
         <is>
@@ -3295,12 +3301,12 @@
         </is>
       </c>
       <c r="U47" s="2" t="n"/>
-      <c r="V47" s="2" t="n"/>
-      <c r="W47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W47" s="2" t="n"/>
       <c r="X47" s="2" t="n"/>
       <c r="Y47" s="2" t="n"/>
       <c r="Z47" s="2" t="n"/>
@@ -3355,12 +3361,12 @@
         </is>
       </c>
       <c r="U48" s="2" t="n"/>
-      <c r="V48" s="2" t="n"/>
-      <c r="W48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W48" s="2" t="n"/>
       <c r="X48" s="2" t="n"/>
       <c r="Y48" s="2" t="inlineStr">
         <is>
@@ -3419,12 +3425,12 @@
         </is>
       </c>
       <c r="U49" s="2" t="n"/>
-      <c r="V49" s="2" t="n"/>
-      <c r="W49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="n"/>
       <c r="X49" s="2" t="n"/>
       <c r="Y49" s="2" t="inlineStr">
         <is>
@@ -3483,12 +3489,12 @@
         </is>
       </c>
       <c r="U50" s="2" t="n"/>
-      <c r="V50" s="2" t="n"/>
-      <c r="W50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="n"/>
       <c r="X50" s="2" t="n"/>
       <c r="Y50" s="2" t="inlineStr">
         <is>
@@ -3543,12 +3549,12 @@
         </is>
       </c>
       <c r="U51" s="2" t="n"/>
-      <c r="V51" s="2" t="n"/>
-      <c r="W51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="n"/>
       <c r="X51" s="2" t="n"/>
       <c r="Y51" s="2" t="n"/>
       <c r="Z51" s="2" t="n"/>
@@ -3599,12 +3605,12 @@
         </is>
       </c>
       <c r="U52" s="2" t="n"/>
-      <c r="V52" s="2" t="n"/>
-      <c r="W52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="n"/>
       <c r="X52" s="2" t="n"/>
       <c r="Y52" s="2" t="n"/>
       <c r="Z52" s="2" t="n"/>
@@ -3659,12 +3665,12 @@
         </is>
       </c>
       <c r="U53" s="2" t="n"/>
-      <c r="V53" s="2" t="n"/>
-      <c r="W53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V53" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W53" s="2" t="n"/>
       <c r="X53" s="2" t="n"/>
       <c r="Y53" s="2" t="inlineStr">
         <is>
@@ -3715,12 +3721,12 @@
         </is>
       </c>
       <c r="U54" s="2" t="n"/>
-      <c r="V54" s="2" t="n"/>
-      <c r="W54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="n"/>
       <c r="X54" s="2" t="n"/>
       <c r="Y54" s="2" t="n"/>
       <c r="Z54" s="2" t="n"/>
@@ -3775,12 +3781,12 @@
         </is>
       </c>
       <c r="U55" s="2" t="n"/>
-      <c r="V55" s="2" t="n"/>
-      <c r="W55" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W55" s="2" t="n"/>
       <c r="X55" s="2" t="n"/>
       <c r="Y55" s="2" t="inlineStr">
         <is>
@@ -3790,60 +3796,60 @@
       <c r="Z55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>BCIO:010121</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>knowledge or skill</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">An expertise of person source that is knowledge or skills held in order to deliver the behaviour change intervention. </t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>expertise of person source</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
-      <c r="J56" s="2" t="n"/>
-      <c r="K56" s="2" t="n"/>
-      <c r="L56" s="2" t="n"/>
-      <c r="M56" s="2" t="n"/>
-      <c r="N56" s="2" t="n"/>
-      <c r="O56" s="2" t="n"/>
-      <c r="P56" s="2" t="n"/>
-      <c r="Q56" s="2" t="inlineStr">
+      <c r="E56" s="3" t="n"/>
+      <c r="F56" s="3" t="n"/>
+      <c r="G56" s="3" t="n"/>
+      <c r="H56" s="3" t="n"/>
+      <c r="I56" s="3" t="n"/>
+      <c r="J56" s="3" t="n"/>
+      <c r="K56" s="3" t="n"/>
+      <c r="L56" s="3" t="n"/>
+      <c r="M56" s="3" t="n"/>
+      <c r="N56" s="3" t="n"/>
+      <c r="O56" s="3" t="n"/>
+      <c r="P56" s="3" t="n"/>
+      <c r="Q56" s="3" t="inlineStr">
         <is>
           <t>trained (if unclear whether pre-existing or acquired)</t>
         </is>
       </c>
-      <c r="R56" s="2" t="n"/>
-      <c r="S56" s="2" t="n"/>
-      <c r="T56" s="2" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="U56" s="2" t="n"/>
-      <c r="V56" s="2" t="n"/>
-      <c r="W56" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="X56" s="2" t="n"/>
-      <c r="Y56" s="2" t="n"/>
-      <c r="Z56" s="2" t="n"/>
+      <c r="R56" s="3" t="n"/>
+      <c r="S56" s="3" t="n"/>
+      <c r="T56" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="U56" s="3" t="n"/>
+      <c r="V56" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="W56" s="3" t="n"/>
+      <c r="X56" s="3" t="n"/>
+      <c r="Y56" s="3" t="n"/>
+      <c r="Z56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3891,12 +3897,12 @@
         </is>
       </c>
       <c r="U57" s="2" t="n"/>
-      <c r="V57" s="2" t="n"/>
-      <c r="W57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="n"/>
       <c r="X57" s="2" t="n"/>
       <c r="Y57" s="2" t="n"/>
       <c r="Z57" s="2" t="n"/>
@@ -3951,12 +3957,12 @@
         </is>
       </c>
       <c r="U58" s="2" t="n"/>
-      <c r="V58" s="2" t="n"/>
-      <c r="W58" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="n"/>
       <c r="X58" s="2" t="n"/>
       <c r="Y58" s="2" t="inlineStr">
         <is>
@@ -4015,12 +4021,12 @@
         </is>
       </c>
       <c r="U59" s="2" t="n"/>
-      <c r="V59" s="2" t="n"/>
-      <c r="W59" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="n"/>
       <c r="X59" s="2" t="n"/>
       <c r="Y59" s="2" t="inlineStr">
         <is>
@@ -4075,12 +4081,12 @@
         </is>
       </c>
       <c r="U60" s="2" t="n"/>
-      <c r="V60" s="2" t="n"/>
-      <c r="W60" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V60" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W60" s="2" t="n"/>
       <c r="X60" s="2" t="n"/>
       <c r="Y60" s="2" t="inlineStr">
         <is>
@@ -4139,12 +4145,12 @@
         </is>
       </c>
       <c r="U61" s="2" t="n"/>
-      <c r="V61" s="2" t="n"/>
-      <c r="W61" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W61" s="2" t="n"/>
       <c r="X61" s="2" t="n"/>
       <c r="Y61" s="2" t="inlineStr">
         <is>
@@ -4199,12 +4205,12 @@
         </is>
       </c>
       <c r="U62" s="2" t="n"/>
-      <c r="V62" s="2" t="n"/>
-      <c r="W62" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V62" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="n"/>
       <c r="X62" s="2" t="n"/>
       <c r="Y62" s="2" t="n"/>
       <c r="Z62" s="2" t="n"/>
@@ -4257,17 +4263,17 @@
       <c r="U63" s="2" t="n"/>
       <c r="V63" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W63" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W63" s="2" t="n"/>
       <c r="X63" s="2" t="n"/>
       <c r="Y63" s="2" t="n"/>
-      <c r="Z63" s="2" t="n"/>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4319,12 +4325,12 @@
         </is>
       </c>
       <c r="U64" s="2" t="n"/>
-      <c r="V64" s="2" t="n"/>
-      <c r="W64" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V64" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W64" s="2" t="n"/>
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="2" t="inlineStr">
         <is>
@@ -4379,12 +4385,12 @@
         </is>
       </c>
       <c r="U65" s="2" t="n"/>
-      <c r="V65" s="2" t="n"/>
-      <c r="W65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V65" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="n"/>
       <c r="X65" s="2" t="n"/>
       <c r="Y65" s="2" t="n"/>
       <c r="Z65" s="2" t="n"/>
@@ -4439,12 +4445,12 @@
         </is>
       </c>
       <c r="U66" s="2" t="n"/>
-      <c r="V66" s="2" t="n"/>
-      <c r="W66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V66" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W66" s="2" t="n"/>
       <c r="X66" s="2" t="n"/>
       <c r="Y66" s="2" t="inlineStr">
         <is>
@@ -4503,12 +4509,12 @@
         </is>
       </c>
       <c r="U67" s="2" t="n"/>
-      <c r="V67" s="2" t="n"/>
-      <c r="W67" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W67" s="2" t="n"/>
       <c r="X67" s="2" t="n"/>
       <c r="Y67" s="2" t="inlineStr">
         <is>
@@ -4567,12 +4573,12 @@
         </is>
       </c>
       <c r="U68" s="2" t="n"/>
-      <c r="V68" s="2" t="n"/>
-      <c r="W68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V68" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W68" s="2" t="n"/>
       <c r="X68" s="2" t="n"/>
       <c r="Y68" s="2" t="inlineStr">
         <is>
@@ -4631,12 +4637,12 @@
         </is>
       </c>
       <c r="U69" s="2" t="n"/>
-      <c r="V69" s="2" t="n"/>
-      <c r="W69" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W69" s="2" t="n"/>
       <c r="X69" s="2" t="n"/>
       <c r="Y69" s="2" t="inlineStr">
         <is>
@@ -4695,12 +4701,12 @@
         </is>
       </c>
       <c r="U70" s="2" t="n"/>
-      <c r="V70" s="2" t="n"/>
-      <c r="W70" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V70" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W70" s="2" t="n"/>
       <c r="X70" s="2" t="n"/>
       <c r="Y70" s="2" t="inlineStr">
         <is>
@@ -4755,12 +4761,12 @@
         </is>
       </c>
       <c r="U71" s="2" t="n"/>
-      <c r="V71" s="2" t="n"/>
-      <c r="W71" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W71" s="2" t="n"/>
       <c r="X71" s="2" t="n"/>
       <c r="Y71" s="2" t="n"/>
       <c r="Z71" s="2" t="n"/>
@@ -4815,12 +4821,12 @@
         </is>
       </c>
       <c r="U72" s="2" t="n"/>
-      <c r="V72" s="2" t="n"/>
-      <c r="W72" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V72" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W72" s="2" t="n"/>
       <c r="X72" s="2" t="n"/>
       <c r="Y72" s="2" t="inlineStr">
         <is>
@@ -4875,12 +4881,12 @@
         </is>
       </c>
       <c r="U73" s="2" t="n"/>
-      <c r="V73" s="2" t="n"/>
-      <c r="W73" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V73" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W73" s="2" t="n"/>
       <c r="X73" s="2" t="n"/>
       <c r="Y73" s="2" t="n"/>
       <c r="Z73" s="2" t="n"/>
@@ -4931,12 +4937,12 @@
         </is>
       </c>
       <c r="U74" s="2" t="n"/>
-      <c r="V74" s="2" t="n"/>
-      <c r="W74" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V74" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W74" s="2" t="n"/>
       <c r="X74" s="2" t="n"/>
       <c r="Y74" s="2" t="n"/>
       <c r="Z74" s="2" t="n"/>
@@ -4991,12 +4997,12 @@
         </is>
       </c>
       <c r="U75" s="2" t="n"/>
-      <c r="V75" s="2" t="n"/>
-      <c r="W75" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V75" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W75" s="2" t="n"/>
       <c r="X75" s="2" t="n"/>
       <c r="Y75" s="2" t="inlineStr">
         <is>
@@ -5051,12 +5057,12 @@
         </is>
       </c>
       <c r="U76" s="2" t="n"/>
-      <c r="V76" s="2" t="n"/>
-      <c r="W76" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V76" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W76" s="2" t="n"/>
       <c r="X76" s="2" t="n"/>
       <c r="Y76" s="2" t="inlineStr">
         <is>
@@ -5115,12 +5121,12 @@
         </is>
       </c>
       <c r="U77" s="2" t="n"/>
-      <c r="V77" s="2" t="n"/>
-      <c r="W77" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V77" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W77" s="2" t="n"/>
       <c r="X77" s="2" t="n"/>
       <c r="Y77" s="2" t="inlineStr">
         <is>
@@ -5179,12 +5185,12 @@
         </is>
       </c>
       <c r="U78" s="2" t="n"/>
-      <c r="V78" s="2" t="n"/>
-      <c r="W78" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V78" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W78" s="2" t="n"/>
       <c r="X78" s="2" t="n"/>
       <c r="Y78" s="2" t="inlineStr">
         <is>
@@ -5239,12 +5245,12 @@
         </is>
       </c>
       <c r="U79" s="2" t="n"/>
-      <c r="V79" s="2" t="n"/>
-      <c r="W79" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V79" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W79" s="2" t="n"/>
       <c r="X79" s="2" t="n"/>
       <c r="Y79" s="2" t="n"/>
       <c r="Z79" s="2" t="n"/>
@@ -5299,12 +5305,12 @@
         </is>
       </c>
       <c r="U80" s="2" t="n"/>
-      <c r="V80" s="2" t="n"/>
-      <c r="W80" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V80" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W80" s="2" t="n"/>
       <c r="X80" s="2" t="n"/>
       <c r="Y80" s="2" t="inlineStr">
         <is>
@@ -5361,17 +5367,17 @@
       <c r="U81" s="2" t="n"/>
       <c r="V81" s="2" t="inlineStr">
         <is>
-          <t>BG; PS</t>
-        </is>
-      </c>
-      <c r="W81" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W81" s="2" t="n"/>
       <c r="X81" s="2" t="n"/>
       <c r="Y81" s="2" t="n"/>
-      <c r="Z81" s="2" t="n"/>
+      <c r="Z81" s="2" t="inlineStr">
+        <is>
+          <t>BG; PS</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5415,12 +5421,12 @@
         </is>
       </c>
       <c r="U82" s="2" t="n"/>
-      <c r="V82" s="2" t="n"/>
-      <c r="W82" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V82" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W82" s="2" t="n"/>
       <c r="X82" s="2" t="n"/>
       <c r="Y82" s="2" t="n"/>
       <c r="Z82" s="2" t="n"/>
@@ -5458,12 +5464,12 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
           <t>RW</t>
-        </is>
-      </c>
-      <c r="W83" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
@@ -5513,12 +5519,12 @@
         </is>
       </c>
       <c r="U84" s="2" t="n"/>
-      <c r="V84" s="2" t="n"/>
-      <c r="W84" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V84" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W84" s="2" t="n"/>
       <c r="X84" s="2" t="n"/>
       <c r="Y84" s="2" t="n"/>
       <c r="Z84" s="2" t="n"/>
@@ -5573,12 +5579,12 @@
         </is>
       </c>
       <c r="U85" s="2" t="n"/>
-      <c r="V85" s="2" t="n"/>
-      <c r="W85" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V85" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W85" s="2" t="n"/>
       <c r="X85" s="2" t="n"/>
       <c r="Y85" s="2" t="inlineStr">
         <is>
@@ -5633,12 +5639,12 @@
         </is>
       </c>
       <c r="U86" s="2" t="n"/>
-      <c r="V86" s="2" t="n"/>
-      <c r="W86" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V86" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W86" s="2" t="n"/>
       <c r="X86" s="2" t="n"/>
       <c r="Y86" s="2" t="n"/>
       <c r="Z86" s="2" t="n"/>
@@ -5689,12 +5695,12 @@
         </is>
       </c>
       <c r="U87" s="2" t="n"/>
-      <c r="V87" s="2" t="n"/>
-      <c r="W87" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V87" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W87" s="2" t="n"/>
       <c r="X87" s="2" t="n"/>
       <c r="Y87" s="2" t="n"/>
       <c r="Z87" s="2" t="n"/>
@@ -5741,12 +5747,12 @@
         </is>
       </c>
       <c r="U88" s="2" t="n"/>
-      <c r="V88" s="2" t="n"/>
-      <c r="W88" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V88" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W88" s="2" t="n"/>
       <c r="X88" s="2" t="n"/>
       <c r="Y88" s="2" t="n"/>
       <c r="Z88" s="2" t="n"/>
@@ -5779,12 +5785,12 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
           <t>AW</t>
-        </is>
-      </c>
-      <c r="W89" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
@@ -5836,17 +5842,17 @@
       <c r="U90" s="2" t="n"/>
       <c r="V90" s="2" t="inlineStr">
         <is>
-          <t>BG</t>
-        </is>
-      </c>
-      <c r="W90" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W90" s="2" t="n"/>
       <c r="X90" s="2" t="n"/>
       <c r="Y90" s="2" t="n"/>
-      <c r="Z90" s="2" t="n"/>
+      <c r="Z90" s="2" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5890,12 +5896,12 @@
         </is>
       </c>
       <c r="U91" s="2" t="n"/>
-      <c r="V91" s="2" t="n"/>
-      <c r="W91" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V91" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W91" s="2" t="n"/>
       <c r="X91" s="2" t="n"/>
       <c r="Y91" s="2" t="n"/>
       <c r="Z91" s="2" t="n"/>
@@ -5950,12 +5956,12 @@
         </is>
       </c>
       <c r="U92" s="2" t="n"/>
-      <c r="V92" s="2" t="n"/>
-      <c r="W92" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V92" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W92" s="2" t="n"/>
       <c r="X92" s="2" t="n"/>
       <c r="Y92" s="2" t="inlineStr">
         <is>
@@ -6006,12 +6012,12 @@
         </is>
       </c>
       <c r="U93" s="2" t="n"/>
-      <c r="V93" s="2" t="n"/>
-      <c r="W93" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V93" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W93" s="2" t="n"/>
       <c r="X93" s="2" t="n"/>
       <c r="Y93" s="2" t="n"/>
       <c r="Z93" s="2" t="n"/>
@@ -6066,12 +6072,12 @@
         </is>
       </c>
       <c r="U94" s="2" t="n"/>
-      <c r="V94" s="2" t="n"/>
-      <c r="W94" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V94" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W94" s="2" t="n"/>
       <c r="X94" s="2" t="n"/>
       <c r="Y94" s="2" t="inlineStr">
         <is>
@@ -6130,12 +6136,12 @@
         </is>
       </c>
       <c r="U95" s="2" t="n"/>
-      <c r="V95" s="2" t="n"/>
-      <c r="W95" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V95" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W95" s="2" t="n"/>
       <c r="X95" s="2" t="n"/>
       <c r="Y95" s="2" t="inlineStr">
         <is>
@@ -6194,12 +6200,12 @@
         </is>
       </c>
       <c r="U96" s="2" t="n"/>
-      <c r="V96" s="2" t="n"/>
-      <c r="W96" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V96" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W96" s="2" t="n"/>
       <c r="X96" s="2" t="n"/>
       <c r="Y96" s="2" t="inlineStr">
         <is>
@@ -6258,12 +6264,12 @@
         </is>
       </c>
       <c r="U97" s="2" t="n"/>
-      <c r="V97" s="2" t="n"/>
-      <c r="W97" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V97" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W97" s="2" t="n"/>
       <c r="X97" s="2" t="n"/>
       <c r="Y97" s="2" t="inlineStr">
         <is>
@@ -6322,12 +6328,12 @@
         </is>
       </c>
       <c r="U98" s="2" t="n"/>
-      <c r="V98" s="2" t="n"/>
-      <c r="W98" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V98" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W98" s="2" t="n"/>
       <c r="X98" s="2" t="n"/>
       <c r="Y98" s="2" t="inlineStr">
         <is>
@@ -6344,17 +6350,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>pre-existing knowledge or skill</t>
+          <t>pre-existing expertise</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>A knowledge or skill that is already possessed by the source which allows them to deliver the behaviour change intervention, including educational level and qualifications.</t>
+          <t>An expertise of person source that is already possessed by the source which allows them to deliver the intervention, including educational level and qualifications.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>knowledge or skill</t>
+          <t>expertise of person source</t>
         </is>
       </c>
       <c r="E99" s="2" t="n"/>
@@ -6382,12 +6388,12 @@
         </is>
       </c>
       <c r="U99" s="2" t="n"/>
-      <c r="V99" s="2" t="n"/>
-      <c r="W99" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V99" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W99" s="2" t="n"/>
       <c r="X99" s="2" t="n"/>
       <c r="Y99" s="2" t="n"/>
       <c r="Z99" s="2" t="n"/>
@@ -6438,12 +6444,12 @@
         </is>
       </c>
       <c r="U100" s="2" t="n"/>
-      <c r="V100" s="2" t="n"/>
-      <c r="W100" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V100" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W100" s="2" t="n"/>
       <c r="X100" s="2" t="n"/>
       <c r="Y100" s="2" t="inlineStr">
         <is>
@@ -6498,12 +6504,12 @@
         </is>
       </c>
       <c r="U101" s="2" t="n"/>
-      <c r="V101" s="2" t="n"/>
-      <c r="W101" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V101" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W101" s="2" t="n"/>
       <c r="X101" s="2" t="n"/>
       <c r="Y101" s="2" t="inlineStr">
         <is>
@@ -6562,12 +6568,12 @@
         </is>
       </c>
       <c r="U102" s="2" t="n"/>
-      <c r="V102" s="2" t="n"/>
-      <c r="W102" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V102" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W102" s="2" t="n"/>
       <c r="X102" s="2" t="n"/>
       <c r="Y102" s="2" t="inlineStr">
         <is>
@@ -6618,12 +6624,12 @@
         </is>
       </c>
       <c r="U103" s="2" t="n"/>
-      <c r="V103" s="2" t="n"/>
-      <c r="W103" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V103" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W103" s="2" t="n"/>
       <c r="X103" s="2" t="n"/>
       <c r="Y103" s="2" t="n"/>
       <c r="Z103" s="2" t="n"/>
@@ -6678,12 +6684,12 @@
         </is>
       </c>
       <c r="U104" s="2" t="n"/>
-      <c r="V104" s="2" t="n"/>
-      <c r="W104" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V104" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W104" s="2" t="n"/>
       <c r="X104" s="2" t="n"/>
       <c r="Y104" s="2" t="inlineStr">
         <is>
@@ -6734,12 +6740,12 @@
         </is>
       </c>
       <c r="U105" s="2" t="n"/>
-      <c r="V105" s="2" t="n"/>
-      <c r="W105" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V105" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W105" s="2" t="n"/>
       <c r="X105" s="2" t="n"/>
       <c r="Y105" s="2" t="n"/>
       <c r="Z105" s="2" t="n"/>
@@ -6794,12 +6800,12 @@
         </is>
       </c>
       <c r="U106" s="2" t="n"/>
-      <c r="V106" s="2" t="n"/>
-      <c r="W106" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V106" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W106" s="2" t="n"/>
       <c r="X106" s="2" t="n"/>
       <c r="Y106" s="2" t="inlineStr">
         <is>
@@ -6854,12 +6860,12 @@
         </is>
       </c>
       <c r="U107" s="2" t="n"/>
-      <c r="V107" s="2" t="n"/>
-      <c r="W107" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V107" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W107" s="2" t="n"/>
       <c r="X107" s="2" t="n"/>
       <c r="Y107" s="2" t="n"/>
       <c r="Z107" s="2" t="n"/>
@@ -6914,12 +6920,12 @@
         </is>
       </c>
       <c r="U108" s="2" t="n"/>
-      <c r="V108" s="2" t="n"/>
-      <c r="W108" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V108" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W108" s="2" t="n"/>
       <c r="X108" s="2" t="n"/>
       <c r="Y108" s="2" t="inlineStr">
         <is>
@@ -6974,12 +6980,12 @@
         </is>
       </c>
       <c r="U109" s="2" t="n"/>
-      <c r="V109" s="2" t="n"/>
-      <c r="W109" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V109" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W109" s="2" t="n"/>
       <c r="X109" s="2" t="n"/>
       <c r="Y109" s="2" t="n"/>
       <c r="Z109" s="2" t="n"/>
@@ -7030,12 +7036,12 @@
         </is>
       </c>
       <c r="U110" s="2" t="n"/>
-      <c r="V110" s="2" t="n"/>
-      <c r="W110" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V110" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W110" s="2" t="n"/>
       <c r="X110" s="2" t="n"/>
       <c r="Y110" s="2" t="n"/>
       <c r="Z110" s="2" t="n"/>
@@ -7090,12 +7096,12 @@
         </is>
       </c>
       <c r="U111" s="2" t="n"/>
-      <c r="V111" s="2" t="n"/>
-      <c r="W111" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V111" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W111" s="2" t="n"/>
       <c r="X111" s="2" t="n"/>
       <c r="Y111" s="2" t="inlineStr">
         <is>
@@ -7146,12 +7152,12 @@
         </is>
       </c>
       <c r="U112" s="2" t="n"/>
-      <c r="V112" s="2" t="n"/>
-      <c r="W112" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V112" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W112" s="2" t="n"/>
       <c r="X112" s="2" t="n"/>
       <c r="Y112" s="2" t="n"/>
       <c r="Z112" s="2" t="n"/>
@@ -7206,12 +7212,12 @@
         </is>
       </c>
       <c r="U113" s="2" t="n"/>
-      <c r="V113" s="2" t="n"/>
-      <c r="W113" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V113" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W113" s="2" t="n"/>
       <c r="X113" s="2" t="n"/>
       <c r="Y113" s="2" t="inlineStr">
         <is>
@@ -7270,12 +7276,12 @@
         </is>
       </c>
       <c r="U114" s="2" t="n"/>
-      <c r="V114" s="2" t="n"/>
-      <c r="W114" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V114" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W114" s="2" t="n"/>
       <c r="X114" s="2" t="n"/>
       <c r="Y114" s="2" t="inlineStr">
         <is>
@@ -7330,12 +7336,12 @@
         </is>
       </c>
       <c r="U115" s="2" t="n"/>
-      <c r="V115" s="2" t="n"/>
-      <c r="W115" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V115" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W115" s="2" t="n"/>
       <c r="X115" s="2" t="n"/>
       <c r="Y115" s="2" t="inlineStr">
         <is>
@@ -7390,12 +7396,12 @@
         </is>
       </c>
       <c r="U116" s="2" t="n"/>
-      <c r="V116" s="2" t="n"/>
-      <c r="W116" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V116" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W116" s="2" t="n"/>
       <c r="X116" s="2" t="n"/>
       <c r="Y116" s="2" t="n"/>
       <c r="Z116" s="2" t="n"/>
@@ -7450,12 +7456,12 @@
         </is>
       </c>
       <c r="U117" s="2" t="n"/>
-      <c r="V117" s="2" t="n"/>
-      <c r="W117" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V117" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W117" s="2" t="n"/>
       <c r="X117" s="2" t="n"/>
       <c r="Y117" s="2" t="inlineStr">
         <is>
@@ -7514,12 +7520,12 @@
         </is>
       </c>
       <c r="U118" s="2" t="n"/>
-      <c r="V118" s="2" t="n"/>
-      <c r="W118" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V118" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W118" s="2" t="n"/>
       <c r="X118" s="2" t="n"/>
       <c r="Y118" s="2" t="inlineStr">
         <is>
@@ -7578,12 +7584,12 @@
         </is>
       </c>
       <c r="U119" s="2" t="n"/>
-      <c r="V119" s="2" t="n"/>
-      <c r="W119" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V119" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W119" s="2" t="n"/>
       <c r="X119" s="2" t="n"/>
       <c r="Y119" s="2" t="inlineStr">
         <is>
@@ -7642,12 +7648,12 @@
         </is>
       </c>
       <c r="U120" s="2" t="n"/>
-      <c r="V120" s="2" t="n"/>
-      <c r="W120" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V120" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W120" s="2" t="n"/>
       <c r="X120" s="2" t="n"/>
       <c r="Y120" s="2" t="inlineStr">
         <is>
@@ -7702,12 +7708,12 @@
         </is>
       </c>
       <c r="U121" s="2" t="n"/>
-      <c r="V121" s="2" t="n"/>
-      <c r="W121" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V121" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W121" s="2" t="n"/>
       <c r="X121" s="2" t="n"/>
       <c r="Y121" s="2" t="n"/>
       <c r="Z121" s="2" t="n"/>
@@ -7754,12 +7760,12 @@
         </is>
       </c>
       <c r="U122" s="2" t="n"/>
-      <c r="V122" s="2" t="n"/>
-      <c r="W122" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V122" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W122" s="2" t="n"/>
       <c r="X122" s="2" t="n"/>
       <c r="Y122" s="2" t="n"/>
       <c r="Z122" s="2" t="n"/>
@@ -7806,12 +7812,12 @@
         </is>
       </c>
       <c r="U123" s="2" t="n"/>
-      <c r="V123" s="2" t="n"/>
-      <c r="W123" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V123" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W123" s="2" t="n"/>
       <c r="X123" s="2" t="n"/>
       <c r="Y123" s="2" t="n"/>
       <c r="Z123" s="2" t="n"/>
@@ -7858,12 +7864,12 @@
         </is>
       </c>
       <c r="U124" s="2" t="n"/>
-      <c r="V124" s="2" t="n"/>
-      <c r="W124" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V124" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W124" s="2" t="n"/>
       <c r="X124" s="2" t="n"/>
       <c r="Y124" s="2" t="n"/>
       <c r="Z124" s="2" t="n"/>
@@ -7918,12 +7924,12 @@
         </is>
       </c>
       <c r="U125" s="2" t="n"/>
-      <c r="V125" s="2" t="n"/>
-      <c r="W125" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V125" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W125" s="2" t="n"/>
       <c r="X125" s="2" t="n"/>
       <c r="Y125" s="2" t="inlineStr">
         <is>
@@ -7982,12 +7988,12 @@
         </is>
       </c>
       <c r="U126" s="2" t="n"/>
-      <c r="V126" s="2" t="n"/>
-      <c r="W126" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V126" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W126" s="2" t="n"/>
       <c r="X126" s="2" t="n"/>
       <c r="Y126" s="2" t="inlineStr">
         <is>
@@ -8046,12 +8052,12 @@
         </is>
       </c>
       <c r="U127" s="2" t="n"/>
-      <c r="V127" s="2" t="n"/>
-      <c r="W127" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V127" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W127" s="2" t="n"/>
       <c r="X127" s="2" t="n"/>
       <c r="Y127" s="2" t="inlineStr">
         <is>
@@ -8110,12 +8116,12 @@
         </is>
       </c>
       <c r="U128" s="2" t="n"/>
-      <c r="V128" s="2" t="n"/>
-      <c r="W128" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V128" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W128" s="2" t="n"/>
       <c r="X128" s="2" t="n"/>
       <c r="Y128" s="2" t="inlineStr">
         <is>
@@ -8170,12 +8176,12 @@
         </is>
       </c>
       <c r="U129" s="2" t="n"/>
-      <c r="V129" s="2" t="n"/>
-      <c r="W129" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V129" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W129" s="2" t="n"/>
       <c r="X129" s="2" t="n"/>
       <c r="Y129" s="2" t="n"/>
       <c r="Z129" s="2" t="n"/>
@@ -8224,17 +8230,17 @@
       <c r="U130" s="2" t="n"/>
       <c r="V130" s="2" t="inlineStr">
         <is>
-          <t>AW</t>
-        </is>
-      </c>
-      <c r="W130" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W130" s="2" t="n"/>
       <c r="X130" s="2" t="n"/>
       <c r="Y130" s="2" t="n"/>
-      <c r="Z130" s="2" t="n"/>
+      <c r="Z130" s="2" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -8286,12 +8292,12 @@
         </is>
       </c>
       <c r="U131" s="2" t="n"/>
-      <c r="V131" s="2" t="n"/>
-      <c r="W131" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V131" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W131" s="2" t="n"/>
       <c r="X131" s="2" t="n"/>
       <c r="Y131" s="2" t="n"/>
       <c r="Z131" s="2" t="n"/>
@@ -8342,12 +8348,12 @@
         </is>
       </c>
       <c r="U132" s="2" t="n"/>
-      <c r="V132" s="2" t="n"/>
-      <c r="W132" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V132" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W132" s="2" t="n"/>
       <c r="X132" s="2" t="n"/>
       <c r="Y132" s="2" t="n"/>
       <c r="Z132" s="2" t="n"/>
@@ -8402,12 +8408,12 @@
         </is>
       </c>
       <c r="U133" s="2" t="n"/>
-      <c r="V133" s="2" t="n"/>
-      <c r="W133" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V133" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W133" s="2" t="n"/>
       <c r="X133" s="2" t="n"/>
       <c r="Y133" s="2" t="inlineStr">
         <is>
@@ -8466,12 +8472,12 @@
         </is>
       </c>
       <c r="U134" s="2" t="n"/>
-      <c r="V134" s="2" t="n"/>
-      <c r="W134" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V134" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W134" s="2" t="n"/>
       <c r="X134" s="2" t="n"/>
       <c r="Y134" s="2" t="inlineStr">
         <is>
@@ -8526,12 +8532,12 @@
         </is>
       </c>
       <c r="U135" s="2" t="n"/>
-      <c r="V135" s="2" t="n"/>
-      <c r="W135" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V135" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W135" s="2" t="n"/>
       <c r="X135" s="2" t="n"/>
       <c r="Y135" s="2" t="inlineStr">
         <is>
@@ -8586,12 +8592,12 @@
         </is>
       </c>
       <c r="U136" s="2" t="n"/>
-      <c r="V136" s="2" t="n"/>
-      <c r="W136" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V136" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W136" s="2" t="n"/>
       <c r="X136" s="2" t="n"/>
       <c r="Y136" s="2" t="n"/>
       <c r="Z136" s="2" t="n"/>
@@ -8646,12 +8652,12 @@
         </is>
       </c>
       <c r="U137" s="2" t="n"/>
-      <c r="V137" s="2" t="n"/>
-      <c r="W137" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V137" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W137" s="2" t="n"/>
       <c r="X137" s="2" t="n"/>
       <c r="Y137" s="2" t="inlineStr">
         <is>
@@ -8710,12 +8716,12 @@
         </is>
       </c>
       <c r="U138" s="2" t="n"/>
-      <c r="V138" s="2" t="n"/>
-      <c r="W138" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V138" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W138" s="2" t="n"/>
       <c r="X138" s="2" t="n"/>
       <c r="Y138" s="2" t="inlineStr">
         <is>
@@ -8766,12 +8772,12 @@
         </is>
       </c>
       <c r="U139" s="2" t="n"/>
-      <c r="V139" s="2" t="n"/>
-      <c r="W139" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V139" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W139" s="2" t="n"/>
       <c r="X139" s="2" t="n"/>
       <c r="Y139" s="2" t="n"/>
       <c r="Z139" s="2" t="n"/>
@@ -8822,12 +8828,12 @@
         </is>
       </c>
       <c r="U140" s="2" t="n"/>
-      <c r="V140" s="2" t="n"/>
-      <c r="W140" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V140" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W140" s="2" t="n"/>
       <c r="X140" s="2" t="n"/>
       <c r="Y140" s="2" t="n"/>
       <c r="Z140" s="2" t="n"/>
@@ -8883,12 +8889,12 @@
         </is>
       </c>
       <c r="U141" s="2" t="n"/>
-      <c r="V141" s="2" t="n"/>
-      <c r="W141" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V141" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W141" s="2" t="n"/>
       <c r="X141" s="2" t="n"/>
       <c r="Y141" s="2" t="inlineStr">
         <is>
@@ -8947,12 +8953,12 @@
         </is>
       </c>
       <c r="U142" s="2" t="n"/>
-      <c r="V142" s="2" t="n"/>
-      <c r="W142" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V142" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W142" s="2" t="n"/>
       <c r="X142" s="2" t="n"/>
       <c r="Y142" s="2" t="inlineStr">
         <is>
@@ -9011,12 +9017,12 @@
         </is>
       </c>
       <c r="U143" s="2" t="n"/>
-      <c r="V143" s="2" t="n"/>
-      <c r="W143" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V143" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W143" s="2" t="n"/>
       <c r="X143" s="2" t="n"/>
       <c r="Y143" s="2" t="inlineStr">
         <is>
@@ -9075,12 +9081,12 @@
         </is>
       </c>
       <c r="U144" s="2" t="n"/>
-      <c r="V144" s="2" t="n"/>
-      <c r="W144" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="V144" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="W144" s="2" t="n"/>
       <c r="X144" s="2" t="n"/>
       <c r="Y144" s="2" t="n"/>
       <c r="Z144" s="2" t="n"/>

</xml_diff>

<commit_message>
Update student or trainee role in bcio_source.xlsx
</commit_message>
<xml_diff>
--- a/Source/bcio_source.xlsx
+++ b/Source/bcio_source.xlsx
@@ -551,12 +551,12 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
+          <t>Definition_ID</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_ID</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -785,12 +785,12 @@
         </is>
       </c>
       <c r="W5" s="2" t="n"/>
-      <c r="X5" s="2" t="n"/>
-      <c r="Y5" s="2" t="inlineStr">
+      <c r="X5" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3258</t>
         </is>
       </c>
+      <c r="Y5" s="2" t="n"/>
       <c r="Z5" s="2" t="n"/>
     </row>
     <row r="6">
@@ -909,12 +909,12 @@
         </is>
       </c>
       <c r="W7" s="2" t="n"/>
-      <c r="X7" s="2" t="n"/>
-      <c r="Y7" s="2" t="inlineStr">
+      <c r="X7" s="2" t="inlineStr">
         <is>
           <t>ISCO: 10</t>
         </is>
       </c>
+      <c r="Y7" s="2" t="n"/>
       <c r="Z7" s="2" t="n"/>
     </row>
     <row r="8">
@@ -973,12 +973,12 @@
         </is>
       </c>
       <c r="W8" s="2" t="n"/>
-      <c r="X8" s="2" t="n"/>
-      <c r="Y8" s="2" t="inlineStr">
+      <c r="X8" s="2" t="inlineStr">
         <is>
           <t>ISCO: 343</t>
         </is>
       </c>
+      <c r="Y8" s="2" t="n"/>
       <c r="Z8" s="2" t="n"/>
     </row>
     <row r="9">
@@ -1037,12 +1037,12 @@
         </is>
       </c>
       <c r="W9" s="2" t="n"/>
-      <c r="X9" s="2" t="n"/>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="X9" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2355</t>
         </is>
       </c>
+      <c r="Y9" s="2" t="n"/>
       <c r="Z9" s="2" t="n"/>
     </row>
     <row r="10">
@@ -1097,12 +1097,12 @@
         </is>
       </c>
       <c r="W10" s="2" t="n"/>
-      <c r="X10" s="2" t="n"/>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="X10" s="2" t="inlineStr">
         <is>
           <t>ISCO: 8</t>
         </is>
       </c>
+      <c r="Y10" s="2" t="n"/>
       <c r="Z10" s="2" t="n"/>
     </row>
     <row r="11">
@@ -1161,12 +1161,12 @@
         </is>
       </c>
       <c r="W11" s="2" t="n"/>
-      <c r="X11" s="2" t="n"/>
-      <c r="Y11" s="2" t="inlineStr">
+      <c r="X11" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3421</t>
         </is>
       </c>
+      <c r="Y11" s="2" t="n"/>
       <c r="Z11" s="2" t="n"/>
     </row>
     <row r="12">
@@ -1225,12 +1225,12 @@
         </is>
       </c>
       <c r="W12" s="2" t="n"/>
-      <c r="X12" s="2" t="n"/>
-      <c r="Y12" s="2" t="inlineStr">
+      <c r="X12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ISCO: 2266 </t>
         </is>
       </c>
+      <c r="Y12" s="2" t="n"/>
       <c r="Z12" s="2" t="n"/>
     </row>
     <row r="13">
@@ -1289,12 +1289,12 @@
         </is>
       </c>
       <c r="W13" s="2" t="n"/>
-      <c r="X13" s="2" t="n"/>
-      <c r="Y13" s="2" t="inlineStr">
+      <c r="X13" s="2" t="inlineStr">
         <is>
           <t>ISCO: 264</t>
         </is>
       </c>
+      <c r="Y13" s="2" t="n"/>
       <c r="Z13" s="2" t="n"/>
     </row>
     <row r="14">
@@ -1457,12 +1457,12 @@
         </is>
       </c>
       <c r="W16" s="2" t="n"/>
-      <c r="X16" s="2" t="n"/>
-      <c r="Y16" s="2" t="inlineStr">
+      <c r="X16" s="2" t="inlineStr">
         <is>
           <t>ISCO: 33</t>
         </is>
       </c>
+      <c r="Y16" s="2" t="n"/>
       <c r="Z16" s="2" t="n"/>
     </row>
     <row r="17">
@@ -1625,12 +1625,12 @@
         </is>
       </c>
       <c r="W19" s="2" t="n"/>
-      <c r="X19" s="2" t="n"/>
-      <c r="Y19" s="2" t="inlineStr">
+      <c r="X19" s="2" t="inlineStr">
         <is>
           <t>ISCO: 5311</t>
         </is>
       </c>
+      <c r="Y19" s="2" t="n"/>
       <c r="Z19" s="2" t="n"/>
     </row>
     <row r="20">
@@ -1745,12 +1745,12 @@
         </is>
       </c>
       <c r="W21" s="2" t="n"/>
-      <c r="X21" s="2" t="n"/>
-      <c r="Y21" s="2" t="inlineStr">
+      <c r="X21" s="2" t="inlineStr">
         <is>
           <t>ISCO: 4</t>
         </is>
       </c>
+      <c r="Y21" s="2" t="n"/>
       <c r="Z21" s="2" t="n"/>
     </row>
     <row r="22">
@@ -1861,12 +1861,12 @@
         </is>
       </c>
       <c r="W23" s="2" t="n"/>
-      <c r="X23" s="2" t="n"/>
-      <c r="Y23" s="2" t="inlineStr">
+      <c r="X23" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3253</t>
         </is>
       </c>
+      <c r="Y23" s="2" t="n"/>
       <c r="Z23" s="2" t="n"/>
     </row>
     <row r="24">
@@ -1925,12 +1925,12 @@
         </is>
       </c>
       <c r="W24" s="2" t="n"/>
-      <c r="X24" s="2" t="n"/>
-      <c r="Y24" s="2" t="inlineStr">
+      <c r="X24" s="2" t="inlineStr">
         <is>
           <t>ISCO: 7</t>
         </is>
       </c>
+      <c r="Y24" s="2" t="n"/>
       <c r="Z24" s="2" t="n"/>
     </row>
     <row r="25">
@@ -1989,12 +1989,12 @@
         </is>
       </c>
       <c r="W25" s="2" t="n"/>
-      <c r="X25" s="2" t="n"/>
-      <c r="Y25" s="2" t="inlineStr">
+      <c r="X25" s="2" t="inlineStr">
         <is>
           <t>ISCO: 265</t>
         </is>
       </c>
+      <c r="Y25" s="2" t="n"/>
       <c r="Z25" s="2" t="n"/>
     </row>
     <row r="26">
@@ -2053,12 +2053,12 @@
         </is>
       </c>
       <c r="W26" s="2" t="n"/>
-      <c r="X26" s="2" t="n"/>
-      <c r="Y26" s="2" t="inlineStr">
+      <c r="X26" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3251</t>
         </is>
       </c>
+      <c r="Y26" s="2" t="n"/>
       <c r="Z26" s="2" t="n"/>
     </row>
     <row r="27">
@@ -2117,12 +2117,12 @@
         </is>
       </c>
       <c r="W27" s="2" t="n"/>
-      <c r="X27" s="2" t="n"/>
-      <c r="Y27" s="2" t="inlineStr">
+      <c r="X27" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2261</t>
         </is>
       </c>
+      <c r="Y27" s="2" t="n"/>
       <c r="Z27" s="2" t="n"/>
     </row>
     <row r="28">
@@ -2181,12 +2181,12 @@
         </is>
       </c>
       <c r="W28" s="2" t="n"/>
-      <c r="X28" s="2" t="n"/>
-      <c r="Y28" s="2" t="inlineStr">
+      <c r="X28" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2265</t>
         </is>
       </c>
+      <c r="Y28" s="2" t="n"/>
       <c r="Z28" s="2" t="n"/>
     </row>
     <row r="29">
@@ -2421,12 +2421,12 @@
         </is>
       </c>
       <c r="W32" s="2" t="n"/>
-      <c r="X32" s="2" t="n"/>
-      <c r="Y32" s="2" t="inlineStr">
+      <c r="X32" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2342</t>
         </is>
       </c>
+      <c r="Y32" s="2" t="n"/>
       <c r="Z32" s="2" t="n"/>
     </row>
     <row r="33">
@@ -2485,12 +2485,12 @@
         </is>
       </c>
       <c r="W33" s="2" t="n"/>
-      <c r="X33" s="2" t="n"/>
-      <c r="Y33" s="2" t="inlineStr">
+      <c r="X33" s="2" t="inlineStr">
         <is>
           <t>ISCO: 9</t>
         </is>
       </c>
+      <c r="Y33" s="2" t="n"/>
       <c r="Z33" s="2" t="n"/>
     </row>
     <row r="34">
@@ -2653,12 +2653,12 @@
         </is>
       </c>
       <c r="W36" s="2" t="n"/>
-      <c r="X36" s="2" t="n"/>
-      <c r="Y36" s="2" t="inlineStr">
+      <c r="X36" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2263</t>
         </is>
       </c>
+      <c r="Y36" s="2" t="n"/>
       <c r="Z36" s="2" t="n"/>
     </row>
     <row r="37">
@@ -2719,12 +2719,12 @@
         </is>
       </c>
       <c r="W37" s="2" t="n"/>
-      <c r="X37" s="2" t="n"/>
-      <c r="Y37" s="2" t="inlineStr">
+      <c r="X37" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3257</t>
         </is>
       </c>
+      <c r="Y37" s="2" t="n"/>
       <c r="Z37" s="2" t="n"/>
     </row>
     <row r="38">
@@ -3071,12 +3071,12 @@
         </is>
       </c>
       <c r="W43" s="2" t="n"/>
-      <c r="X43" s="2" t="n"/>
-      <c r="Y43" s="2" t="inlineStr">
+      <c r="X43" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3423</t>
         </is>
       </c>
+      <c r="Y43" s="2" t="n"/>
       <c r="Z43" s="2" t="n"/>
     </row>
     <row r="44">
@@ -3299,12 +3299,12 @@
         </is>
       </c>
       <c r="W47" s="2" t="n"/>
-      <c r="X47" s="2" t="n"/>
-      <c r="Y47" s="2" t="inlineStr">
+      <c r="X47" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2211</t>
         </is>
       </c>
+      <c r="Y47" s="2" t="n"/>
       <c r="Z47" s="2" t="n"/>
     </row>
     <row r="48">
@@ -3419,12 +3419,12 @@
         </is>
       </c>
       <c r="W49" s="2" t="n"/>
-      <c r="X49" s="2" t="n"/>
-      <c r="Y49" s="2" t="inlineStr">
+      <c r="X49" s="2" t="inlineStr">
         <is>
           <t>ISCO: 32</t>
         </is>
       </c>
+      <c r="Y49" s="2" t="n"/>
       <c r="Z49" s="2" t="n"/>
     </row>
     <row r="50">
@@ -3483,12 +3483,12 @@
         </is>
       </c>
       <c r="W50" s="2" t="n"/>
-      <c r="X50" s="2" t="n"/>
-      <c r="Y50" s="2" t="inlineStr">
+      <c r="X50" s="2" t="inlineStr">
         <is>
           <t>ISCO: 5321</t>
         </is>
       </c>
+      <c r="Y50" s="2" t="n"/>
       <c r="Z50" s="2" t="n"/>
     </row>
     <row r="51">
@@ -3547,12 +3547,12 @@
         </is>
       </c>
       <c r="W51" s="2" t="n"/>
-      <c r="X51" s="2" t="n"/>
-      <c r="Y51" s="2" t="inlineStr">
+      <c r="X51" s="2" t="inlineStr">
         <is>
           <t>ISCO: 22</t>
         </is>
       </c>
+      <c r="Y51" s="2" t="n"/>
       <c r="Z51" s="2" t="n"/>
     </row>
     <row r="52">
@@ -3723,12 +3723,12 @@
         </is>
       </c>
       <c r="W54" s="2" t="n"/>
-      <c r="X54" s="2" t="n"/>
-      <c r="Y54" s="2" t="inlineStr">
+      <c r="X54" s="2" t="inlineStr">
         <is>
           <t>ISCO: 5322</t>
         </is>
       </c>
+      <c r="Y54" s="2" t="n"/>
       <c r="Z54" s="2" t="n"/>
     </row>
     <row r="55">
@@ -3839,12 +3839,12 @@
         </is>
       </c>
       <c r="W56" s="2" t="n"/>
-      <c r="X56" s="2" t="n"/>
-      <c r="Y56" s="2" t="inlineStr">
+      <c r="X56" s="2" t="inlineStr">
         <is>
           <t>ISCO: 35</t>
         </is>
       </c>
+      <c r="Y56" s="2" t="n"/>
       <c r="Z56" s="2" t="n"/>
     </row>
     <row r="57">
@@ -4015,12 +4015,12 @@
         </is>
       </c>
       <c r="W59" s="2" t="n"/>
-      <c r="X59" s="2" t="n"/>
-      <c r="Y59" s="2" t="inlineStr">
+      <c r="X59" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3411</t>
         </is>
       </c>
+      <c r="Y59" s="2" t="n"/>
       <c r="Z59" s="2" t="n"/>
     </row>
     <row r="60">
@@ -4079,12 +4079,12 @@
         </is>
       </c>
       <c r="W60" s="2" t="n"/>
-      <c r="X60" s="2" t="n"/>
-      <c r="Y60" s="2" t="inlineStr">
+      <c r="X60" s="2" t="inlineStr">
         <is>
           <t>ISCO: 261</t>
         </is>
       </c>
+      <c r="Y60" s="2" t="n"/>
       <c r="Z60" s="2" t="n"/>
     </row>
     <row r="61">
@@ -4139,12 +4139,12 @@
         </is>
       </c>
       <c r="W61" s="2" t="n"/>
-      <c r="X61" s="2" t="n"/>
-      <c r="Y61" s="2" t="inlineStr">
+      <c r="X61" s="2" t="inlineStr">
         <is>
           <t>ISCO: 26</t>
         </is>
       </c>
+      <c r="Y61" s="2" t="n"/>
       <c r="Z61" s="2" t="n"/>
     </row>
     <row r="62">
@@ -4203,12 +4203,12 @@
         </is>
       </c>
       <c r="W62" s="2" t="n"/>
-      <c r="X62" s="2" t="n"/>
-      <c r="Y62" s="2" t="inlineStr">
+      <c r="X62" s="2" t="inlineStr">
         <is>
           <t>ISCO: 262</t>
         </is>
       </c>
+      <c r="Y62" s="2" t="n"/>
       <c r="Z62" s="2" t="n"/>
     </row>
     <row r="63">
@@ -4383,12 +4383,12 @@
         </is>
       </c>
       <c r="W65" s="2" t="n"/>
-      <c r="X65" s="2" t="n"/>
-      <c r="Y65" s="2" t="inlineStr">
+      <c r="X65" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ISCO: 1 </t>
         </is>
       </c>
+      <c r="Y65" s="2" t="n"/>
       <c r="Z65" s="2" t="n"/>
     </row>
     <row r="66">
@@ -4503,12 +4503,12 @@
         </is>
       </c>
       <c r="W67" s="2" t="n"/>
-      <c r="X67" s="2" t="n"/>
-      <c r="Y67" s="2" t="inlineStr">
+      <c r="X67" s="2" t="inlineStr">
         <is>
           <t>ISCO: 321</t>
         </is>
       </c>
+      <c r="Y67" s="2" t="n"/>
       <c r="Z67" s="2" t="n"/>
     </row>
     <row r="68">
@@ -4567,12 +4567,12 @@
         </is>
       </c>
       <c r="W68" s="2" t="n"/>
-      <c r="X68" s="2" t="n"/>
-      <c r="Y68" s="2" t="inlineStr">
+      <c r="X68" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3256</t>
         </is>
       </c>
+      <c r="Y68" s="2" t="n"/>
       <c r="Z68" s="2" t="n"/>
     </row>
     <row r="69">
@@ -4631,12 +4631,12 @@
         </is>
       </c>
       <c r="W69" s="2" t="n"/>
-      <c r="X69" s="2" t="n"/>
-      <c r="Y69" s="2" t="inlineStr">
+      <c r="X69" s="2" t="inlineStr">
         <is>
           <t>ISCO: 221</t>
         </is>
       </c>
+      <c r="Y69" s="2" t="n"/>
       <c r="Z69" s="2" t="n"/>
     </row>
     <row r="70">
@@ -4695,12 +4695,12 @@
         </is>
       </c>
       <c r="W70" s="2" t="n"/>
-      <c r="X70" s="2" t="n"/>
-      <c r="Y70" s="2" t="inlineStr">
+      <c r="X70" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3222</t>
         </is>
       </c>
+      <c r="Y70" s="2" t="n"/>
       <c r="Z70" s="2" t="n"/>
     </row>
     <row r="71">
@@ -4759,12 +4759,12 @@
         </is>
       </c>
       <c r="W71" s="2" t="n"/>
-      <c r="X71" s="2" t="n"/>
-      <c r="Y71" s="2" t="inlineStr">
+      <c r="X71" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2222</t>
         </is>
       </c>
+      <c r="Y71" s="2" t="n"/>
       <c r="Z71" s="2" t="n"/>
     </row>
     <row r="72">
@@ -4879,12 +4879,12 @@
         </is>
       </c>
       <c r="W73" s="2" t="n"/>
-      <c r="X73" s="2" t="n"/>
-      <c r="Y73" s="2" t="inlineStr">
+      <c r="X73" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2354</t>
         </is>
       </c>
+      <c r="Y73" s="2" t="n"/>
       <c r="Z73" s="2" t="n"/>
     </row>
     <row r="74">
@@ -5055,12 +5055,12 @@
         </is>
       </c>
       <c r="W76" s="2" t="n"/>
-      <c r="X76" s="2" t="n"/>
-      <c r="Y76" s="2" t="inlineStr">
+      <c r="X76" s="2" t="inlineStr">
         <is>
           <t>ISCO: 322</t>
         </is>
       </c>
+      <c r="Y76" s="2" t="n"/>
       <c r="Z76" s="2" t="n"/>
     </row>
     <row r="77">
@@ -5115,12 +5115,12 @@
         </is>
       </c>
       <c r="W77" s="2" t="n"/>
-      <c r="X77" s="2" t="n"/>
-      <c r="Y77" s="2" t="inlineStr">
+      <c r="X77" s="2" t="inlineStr">
         <is>
           <t>ISCO: 222</t>
         </is>
       </c>
+      <c r="Y77" s="2" t="n"/>
       <c r="Z77" s="2" t="n"/>
     </row>
     <row r="78">
@@ -5179,12 +5179,12 @@
         </is>
       </c>
       <c r="W78" s="2" t="n"/>
-      <c r="X78" s="2" t="n"/>
-      <c r="Y78" s="2" t="inlineStr">
+      <c r="X78" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3221</t>
         </is>
       </c>
+      <c r="Y78" s="2" t="n"/>
       <c r="Z78" s="2" t="n"/>
     </row>
     <row r="79">
@@ -5243,12 +5243,12 @@
         </is>
       </c>
       <c r="W79" s="2" t="n"/>
-      <c r="X79" s="2" t="n"/>
-      <c r="Y79" s="2" t="inlineStr">
+      <c r="X79" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2221</t>
         </is>
       </c>
+      <c r="Y79" s="2" t="n"/>
       <c r="Z79" s="2" t="n"/>
     </row>
     <row r="80">
@@ -5363,12 +5363,12 @@
         </is>
       </c>
       <c r="W81" s="2" t="n"/>
-      <c r="X81" s="2" t="n"/>
-      <c r="Y81" s="2" t="inlineStr">
+      <c r="X81" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2267</t>
         </is>
       </c>
+      <c r="Y81" s="2" t="n"/>
       <c r="Z81" s="2" t="n"/>
     </row>
     <row r="82">
@@ -5637,12 +5637,12 @@
         </is>
       </c>
       <c r="W86" s="2" t="n"/>
-      <c r="X86" s="2" t="n"/>
-      <c r="Y86" s="2" t="inlineStr">
+      <c r="X86" s="2" t="inlineStr">
         <is>
           <t>ISCO: 224</t>
         </is>
       </c>
+      <c r="Y86" s="2" t="n"/>
       <c r="Z86" s="2" t="n"/>
     </row>
     <row r="87">
@@ -6014,12 +6014,12 @@
         </is>
       </c>
       <c r="W93" s="2" t="n"/>
-      <c r="X93" s="2" t="n"/>
-      <c r="Y93" s="2" t="inlineStr">
+      <c r="X93" s="2" t="inlineStr">
         <is>
           <t>ISCO: 53</t>
         </is>
       </c>
+      <c r="Y93" s="2" t="n"/>
       <c r="Z93" s="2" t="n"/>
     </row>
     <row r="94">
@@ -6182,12 +6182,12 @@
         </is>
       </c>
       <c r="W96" s="2" t="n"/>
-      <c r="X96" s="2" t="n"/>
-      <c r="Y96" s="2" t="inlineStr">
+      <c r="X96" s="2" t="inlineStr">
         <is>
           <t>ISCO: 51</t>
         </is>
       </c>
+      <c r="Y96" s="2" t="n"/>
       <c r="Z96" s="2" t="n"/>
     </row>
     <row r="97">
@@ -6246,12 +6246,12 @@
         </is>
       </c>
       <c r="W97" s="2" t="n"/>
-      <c r="X97" s="2" t="n"/>
-      <c r="Y97" s="2" t="inlineStr">
+      <c r="X97" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2262</t>
         </is>
       </c>
+      <c r="Y97" s="2" t="n"/>
       <c r="Z97" s="2" t="n"/>
     </row>
     <row r="98">
@@ -6310,12 +6310,12 @@
         </is>
       </c>
       <c r="W98" s="2" t="n"/>
-      <c r="X98" s="2" t="n"/>
-      <c r="Y98" s="2" t="inlineStr">
+      <c r="X98" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2264</t>
         </is>
       </c>
+      <c r="Y98" s="2" t="n"/>
       <c r="Z98" s="2" t="n"/>
     </row>
     <row r="99">
@@ -6374,12 +6374,12 @@
         </is>
       </c>
       <c r="W99" s="2" t="n"/>
-      <c r="X99" s="2" t="n"/>
-      <c r="Y99" s="2" t="inlineStr">
+      <c r="X99" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3255</t>
         </is>
       </c>
+      <c r="Y99" s="2" t="n"/>
       <c r="Z99" s="2" t="n"/>
     </row>
     <row r="100">
@@ -6438,12 +6438,12 @@
         </is>
       </c>
       <c r="W100" s="2" t="n"/>
-      <c r="X100" s="2" t="n"/>
-      <c r="Y100" s="2" t="inlineStr">
+      <c r="X100" s="2" t="inlineStr">
         <is>
           <t>ISCO: 8</t>
         </is>
       </c>
+      <c r="Y100" s="2" t="n"/>
       <c r="Z100" s="2" t="n"/>
     </row>
     <row r="101">
@@ -6554,12 +6554,12 @@
         </is>
       </c>
       <c r="W102" s="2" t="n"/>
-      <c r="X102" s="2" t="n"/>
-      <c r="Y102" s="2" t="inlineStr">
+      <c r="X102" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2341</t>
         </is>
       </c>
+      <c r="Y102" s="2" t="n"/>
       <c r="Z102" s="2" t="n"/>
     </row>
     <row r="103">
@@ -6614,12 +6614,12 @@
         </is>
       </c>
       <c r="W103" s="2" t="n"/>
-      <c r="X103" s="2" t="n"/>
-      <c r="Y103" s="2" t="inlineStr">
+      <c r="X103" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2</t>
         </is>
       </c>
+      <c r="Y103" s="2" t="n"/>
       <c r="Z103" s="2" t="n"/>
     </row>
     <row r="104">
@@ -6678,12 +6678,12 @@
         </is>
       </c>
       <c r="W104" s="2" t="n"/>
-      <c r="X104" s="2" t="n"/>
-      <c r="Y104" s="2" t="inlineStr">
+      <c r="X104" s="2" t="inlineStr">
         <is>
           <t>ISCO: 54</t>
         </is>
       </c>
+      <c r="Y104" s="2" t="n"/>
       <c r="Z104" s="2" t="n"/>
     </row>
     <row r="105">
@@ -6794,12 +6794,12 @@
         </is>
       </c>
       <c r="W106" s="2" t="n"/>
-      <c r="X106" s="2" t="n"/>
-      <c r="Y106" s="2" t="inlineStr">
+      <c r="X106" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2634</t>
         </is>
       </c>
+      <c r="Y106" s="2" t="n"/>
       <c r="Z106" s="2" t="n"/>
     </row>
     <row r="107">
@@ -6910,12 +6910,12 @@
         </is>
       </c>
       <c r="W108" s="2" t="n"/>
-      <c r="X108" s="2" t="n"/>
-      <c r="Y108" s="2" t="inlineStr">
+      <c r="X108" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3413</t>
         </is>
       </c>
+      <c r="Y108" s="2" t="n"/>
       <c r="Z108" s="2" t="n"/>
     </row>
     <row r="109">
@@ -7030,12 +7030,12 @@
         </is>
       </c>
       <c r="W110" s="2" t="n"/>
-      <c r="X110" s="2" t="n"/>
-      <c r="Y110" s="2" t="inlineStr">
+      <c r="X110" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2636</t>
         </is>
       </c>
+      <c r="Y110" s="2" t="n"/>
       <c r="Z110" s="2" t="n"/>
     </row>
     <row r="111">
@@ -7206,12 +7206,12 @@
         </is>
       </c>
       <c r="W113" s="2" t="n"/>
-      <c r="X113" s="2" t="n"/>
-      <c r="Y113" s="2" t="inlineStr">
+      <c r="X113" s="2" t="inlineStr">
         <is>
           <t>ISCO: 52</t>
         </is>
       </c>
+      <c r="Y113" s="2" t="n"/>
       <c r="Z113" s="2" t="n"/>
     </row>
     <row r="114">
@@ -7322,12 +7322,12 @@
         </is>
       </c>
       <c r="W115" s="2" t="n"/>
-      <c r="X115" s="2" t="n"/>
-      <c r="Y115" s="2" t="inlineStr">
+      <c r="X115" s="2" t="inlineStr">
         <is>
           <t>ISCO: 21</t>
         </is>
       </c>
+      <c r="Y115" s="2" t="n"/>
       <c r="Z115" s="2" t="n"/>
     </row>
     <row r="116">
@@ -7386,12 +7386,12 @@
         </is>
       </c>
       <c r="W116" s="2" t="n"/>
-      <c r="X116" s="2" t="n"/>
-      <c r="Y116" s="2" t="inlineStr">
+      <c r="X116" s="2" t="inlineStr">
         <is>
           <t>ISCO: 233</t>
         </is>
       </c>
+      <c r="Y116" s="2" t="n"/>
       <c r="Z116" s="2" t="n"/>
     </row>
     <row r="117">
@@ -7446,12 +7446,12 @@
         </is>
       </c>
       <c r="W117" s="2" t="n"/>
-      <c r="X117" s="2" t="n"/>
-      <c r="Y117" s="2" t="inlineStr">
+      <c r="X117" s="2" t="inlineStr">
         <is>
           <t>ISCO: 5</t>
         </is>
       </c>
+      <c r="Y117" s="2" t="n"/>
       <c r="Z117" s="2" t="n"/>
     </row>
     <row r="118">
@@ -7566,12 +7566,12 @@
         </is>
       </c>
       <c r="W119" s="2" t="n"/>
-      <c r="X119" s="2" t="n"/>
-      <c r="Y119" s="2" t="inlineStr">
+      <c r="X119" s="2" t="inlineStr">
         <is>
           <t>ISCO: 6</t>
         </is>
       </c>
+      <c r="Y119" s="2" t="n"/>
       <c r="Z119" s="2" t="n"/>
     </row>
     <row r="120">
@@ -7630,12 +7630,12 @@
         </is>
       </c>
       <c r="W120" s="2" t="n"/>
-      <c r="X120" s="2" t="n"/>
-      <c r="Y120" s="2" t="inlineStr">
+      <c r="X120" s="2" t="inlineStr">
         <is>
           <t>ISCO: 263</t>
         </is>
       </c>
+      <c r="Y120" s="2" t="n"/>
       <c r="Z120" s="2" t="n"/>
     </row>
     <row r="121">
@@ -7694,12 +7694,12 @@
         </is>
       </c>
       <c r="W121" s="2" t="n"/>
-      <c r="X121" s="2" t="n"/>
-      <c r="Y121" s="2" t="inlineStr">
+      <c r="X121" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2635</t>
         </is>
       </c>
+      <c r="Y121" s="2" t="n"/>
       <c r="Z121" s="2" t="n"/>
     </row>
     <row r="122">
@@ -7758,12 +7758,12 @@
         </is>
       </c>
       <c r="W122" s="2" t="n"/>
-      <c r="X122" s="2" t="n"/>
-      <c r="Y122" s="2" t="inlineStr">
+      <c r="X122" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3412</t>
         </is>
       </c>
+      <c r="Y122" s="2" t="n"/>
       <c r="Z122" s="2" t="n"/>
     </row>
     <row r="123">
@@ -8034,12 +8034,12 @@
         </is>
       </c>
       <c r="W127" s="2" t="n"/>
-      <c r="X127" s="2" t="n"/>
-      <c r="Y127" s="2" t="inlineStr">
+      <c r="X127" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2352</t>
         </is>
       </c>
+      <c r="Y127" s="2" t="n"/>
       <c r="Z127" s="2" t="n"/>
     </row>
     <row r="128">
@@ -8098,12 +8098,12 @@
         </is>
       </c>
       <c r="W128" s="2" t="n"/>
-      <c r="X128" s="2" t="n"/>
-      <c r="Y128" s="2" t="inlineStr">
+      <c r="X128" s="2" t="inlineStr">
         <is>
           <t>ISCO: 2212</t>
         </is>
       </c>
+      <c r="Y128" s="2" t="n"/>
       <c r="Z128" s="2" t="n"/>
     </row>
     <row r="129">
@@ -8162,12 +8162,12 @@
         </is>
       </c>
       <c r="W129" s="2" t="n"/>
-      <c r="X129" s="2" t="n"/>
-      <c r="Y129" s="2" t="inlineStr">
+      <c r="X129" s="2" t="inlineStr">
         <is>
           <t>ISCO: 342</t>
         </is>
       </c>
+      <c r="Y129" s="2" t="n"/>
       <c r="Z129" s="2" t="n"/>
     </row>
     <row r="130">
@@ -8226,12 +8226,12 @@
         </is>
       </c>
       <c r="W130" s="2" t="n"/>
-      <c r="X130" s="2" t="n"/>
-      <c r="Y130" s="2" t="inlineStr">
+      <c r="X130" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3422</t>
         </is>
       </c>
+      <c r="Y130" s="2" t="n"/>
       <c r="Z130" s="2" t="n"/>
     </row>
     <row r="131">
@@ -8303,12 +8303,12 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>A role which inheres in a person and is realised by being enrolled in an educational institution or a formal programme of professional training.</t>
+          <t>A personal role which inheres in a person and is realised by being enrolled in an educational institution or a formal programme of professional training.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>personal role</t>
         </is>
       </c>
       <c r="E132" s="2" t="n"/>
@@ -8518,12 +8518,12 @@
         </is>
       </c>
       <c r="W135" s="2" t="n"/>
-      <c r="X135" s="2" t="n"/>
-      <c r="Y135" s="2" t="inlineStr">
+      <c r="X135" s="2" t="inlineStr">
         <is>
           <t>ISCO: 5312</t>
         </is>
       </c>
+      <c r="Y135" s="2" t="n"/>
       <c r="Z135" s="2" t="n"/>
     </row>
     <row r="136">
@@ -8582,12 +8582,12 @@
         </is>
       </c>
       <c r="W136" s="2" t="n"/>
-      <c r="X136" s="2" t="n"/>
-      <c r="Y136" s="2" t="inlineStr">
+      <c r="X136" s="2" t="inlineStr">
         <is>
           <t>ISCO: 23</t>
         </is>
       </c>
+      <c r="Y136" s="2" t="n"/>
       <c r="Z136" s="2" t="n"/>
     </row>
     <row r="137">
@@ -8642,12 +8642,12 @@
         </is>
       </c>
       <c r="W137" s="2" t="n"/>
-      <c r="X137" s="2" t="n"/>
-      <c r="Y137" s="2" t="inlineStr">
+      <c r="X137" s="2" t="inlineStr">
         <is>
           <t>ISCO: 3</t>
         </is>
       </c>
+      <c r="Y137" s="2" t="n"/>
       <c r="Z137" s="2" t="n"/>
     </row>
     <row r="138">
@@ -8762,12 +8762,12 @@
         </is>
       </c>
       <c r="W139" s="2" t="n"/>
-      <c r="X139" s="2" t="n"/>
-      <c r="Y139" s="2" t="inlineStr">
+      <c r="X139" s="2" t="inlineStr">
         <is>
           <t>ISCO: 323</t>
         </is>
       </c>
+      <c r="Y139" s="2" t="n"/>
       <c r="Z139" s="2" t="n"/>
     </row>
     <row r="140">
@@ -8826,12 +8826,12 @@
         </is>
       </c>
       <c r="W140" s="2" t="n"/>
-      <c r="X140" s="2" t="n"/>
-      <c r="Y140" s="2" t="inlineStr">
+      <c r="X140" s="2" t="inlineStr">
         <is>
           <t>ISCO: 223</t>
         </is>
       </c>
+      <c r="Y140" s="2" t="n"/>
       <c r="Z140" s="2" t="n"/>
     </row>
     <row r="141">
@@ -8999,12 +8999,12 @@
         </is>
       </c>
       <c r="W143" s="2" t="n"/>
-      <c r="X143" s="2" t="n"/>
-      <c r="Y143" s="2" t="inlineStr">
+      <c r="X143" s="2" t="inlineStr">
         <is>
           <t>ISCO: 231</t>
         </is>
       </c>
+      <c r="Y143" s="2" t="n"/>
       <c r="Z143" s="2" t="n"/>
     </row>
     <row r="144">
@@ -9063,12 +9063,12 @@
         </is>
       </c>
       <c r="W144" s="2" t="n"/>
-      <c r="X144" s="2" t="n"/>
-      <c r="Y144" s="2" t="inlineStr">
+      <c r="X144" s="2" t="inlineStr">
         <is>
           <t>ISCO: 225</t>
         </is>
       </c>
+      <c r="Y144" s="2" t="n"/>
       <c r="Z144" s="2" t="n"/>
     </row>
     <row r="145">
@@ -9127,12 +9127,12 @@
         </is>
       </c>
       <c r="W145" s="2" t="n"/>
-      <c r="X145" s="2" t="n"/>
-      <c r="Y145" s="2" t="inlineStr">
+      <c r="X145" s="2" t="inlineStr">
         <is>
           <t>ISCO: 232</t>
         </is>
       </c>
+      <c r="Y145" s="2" t="n"/>
       <c r="Z145" s="2" t="n"/>
     </row>
     <row r="146">

</xml_diff>